<commit_message>
Contest 1 KKR vs RCB
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D53D0A5-B1D2-FC40-9A4A-C126ACEE13A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB180D7C-2726-BC4F-AF52-1938E32B45A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -1454,51 +1454,69 @@
       <c r="C14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="3" t="str">
+      <c r="D14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="G14" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>70</v>
+      </c>
+      <c r="G14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H14" s="1"/>
-      <c r="J14" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H14" s="1">
+        <v>90</v>
+      </c>
+      <c r="J14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K14" s="1"/>
-      <c r="M14" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K14" s="1">
+        <v>50</v>
+      </c>
+      <c r="M14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N14" s="1"/>
-      <c r="P14" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N14" s="1">
+        <v>40</v>
+      </c>
+      <c r="P14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q14" s="1"/>
-      <c r="S14" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>80</v>
+      </c>
+      <c r="S14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T14" s="1"/>
-      <c r="V14" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="T14" s="1">
+        <v>0</v>
+      </c>
+      <c r="V14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W14" s="1"/>
-      <c r="Y14" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W14" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z14" s="1"/>
-      <c r="AB14" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Z14" s="1">
+        <v>60</v>
+      </c>
+      <c r="AB14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14,$AC14), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC14" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="AC14" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
@@ -2163,49 +2181,49 @@
       </c>
       <c r="H27" s="10">
         <f>SUM(G14:G24)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K27" s="10">
         <f>SUM(J14:J24)</f>
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N27" s="10">
         <f>SUM(M14:M24)</f>
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="P27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q27" s="10">
         <f>SUM(P14:P24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T27" s="10">
         <f>SUM(S14:S24)</f>
-        <v>0</v>
+        <v>-25</v>
       </c>
       <c r="V27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W27" s="10">
         <f>SUM(V14:V24)</f>
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="Y27" s="26" t="s">
         <v>7</v>
       </c>
       <c r="Z27" s="10">
         <f>SUM(Y14:Y24)</f>
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="AA27" s="25"/>
       <c r="AB27" s="26" t="s">
@@ -2213,7 +2231,7 @@
       </c>
       <c r="AC27" s="10">
         <f>SUM(AB14:AB24)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="AD27" s="1">
         <f>SUM(E27,H27,K27,N27,Q27,T27,W27,Z27,AC27)</f>

</xml_diff>

<commit_message>
Contest 3 CSK vs MI
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB180D7C-2726-BC4F-AF52-1938E32B45A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBF5628-9F67-094D-8D64-13FD6CA66C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -1528,51 +1528,69 @@
       <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="3" t="str">
+      <c r="D15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E15" s="1"/>
-      <c r="G15" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E15" s="1">
+        <v>80</v>
+      </c>
+      <c r="G15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="J15" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H15" s="1">
+        <v>60</v>
+      </c>
+      <c r="J15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K15" s="1"/>
-      <c r="M15" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K15" s="1">
+        <v>40</v>
+      </c>
+      <c r="M15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N15" s="1"/>
-      <c r="P15" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N15" s="1">
+        <v>30</v>
+      </c>
+      <c r="P15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q15" s="1"/>
-      <c r="S15" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>0</v>
+      </c>
+      <c r="S15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T15" s="1"/>
-      <c r="V15" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T15" s="1">
+        <v>90</v>
+      </c>
+      <c r="V15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W15" s="1"/>
-      <c r="Y15" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W15" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z15" s="1"/>
-      <c r="AB15" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Z15" s="1">
+        <v>50</v>
+      </c>
+      <c r="AB15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15,$AC15), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC15" s="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
@@ -1584,51 +1602,69 @@
       <c r="C16" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="3" t="str">
+      <c r="D16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E16" s="1"/>
-      <c r="G16" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>70</v>
+      </c>
+      <c r="G16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H16" s="1"/>
-      <c r="J16" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K16" s="1"/>
-      <c r="M16" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K16" s="1">
+        <v>80</v>
+      </c>
+      <c r="M16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N16" s="1"/>
-      <c r="P16" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N16" s="1">
+        <v>100</v>
+      </c>
+      <c r="P16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q16" s="1"/>
-      <c r="S16" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>50</v>
+      </c>
+      <c r="S16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T16" s="1"/>
-      <c r="V16" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T16" s="1">
+        <v>90</v>
+      </c>
+      <c r="V16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W16" s="1"/>
-      <c r="Y16" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W16" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z16" s="1"/>
-      <c r="AB16" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Z16" s="1">
+        <v>60</v>
+      </c>
+      <c r="AB16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16,$AC16), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC16" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="AC16" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
@@ -2174,56 +2210,56 @@
       </c>
       <c r="E27" s="10">
         <f>SUM(D14:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H27" s="10">
         <f>SUM(G14:G24)</f>
-        <v>20</v>
+        <v>-10</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K27" s="10">
         <f>SUM(J14:J24)</f>
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N27" s="10">
         <f>SUM(M14:M24)</f>
-        <v>-15</v>
+        <v>15</v>
       </c>
       <c r="P27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q27" s="10">
         <f>SUM(P14:P24)</f>
-        <v>5</v>
+        <v>-30</v>
       </c>
       <c r="S27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T27" s="10">
         <f>SUM(S14:S24)</f>
-        <v>-25</v>
+        <v>15</v>
       </c>
       <c r="V27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W27" s="10">
         <f>SUM(V14:V24)</f>
-        <v>-20</v>
+        <v>15</v>
       </c>
       <c r="Y27" s="26" t="s">
         <v>7</v>
       </c>
       <c r="Z27" s="10">
         <f>SUM(Y14:Y24)</f>
-        <v>-5</v>
+        <v>-20</v>
       </c>
       <c r="AA27" s="25"/>
       <c r="AB27" s="26" t="s">
@@ -2231,7 +2267,7 @@
       </c>
       <c r="AC27" s="10">
         <f>SUM(AB14:AB24)</f>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="AD27" s="1">
         <f>SUM(E27,H27,K27,N27,Q27,T27,W27,Z27,AC27)</f>

</xml_diff>

<commit_message>
Contest 4 DC vs LSG
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBF5628-9F67-094D-8D64-13FD6CA66C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{069CB805-D01F-8F40-A854-389F6F17706D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -1676,51 +1676,69 @@
       <c r="C17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="3" t="str">
+      <c r="D17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="G17" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="E17" s="1">
+        <v>30</v>
+      </c>
+      <c r="G17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H17" s="1"/>
-      <c r="J17" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H17" s="1">
+        <v>80</v>
+      </c>
+      <c r="J17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K17" s="1"/>
-      <c r="M17" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>70</v>
+      </c>
+      <c r="M17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N17" s="1"/>
-      <c r="P17" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N17" s="1">
+        <v>40</v>
+      </c>
+      <c r="P17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q17" s="1"/>
-      <c r="S17" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>60</v>
+      </c>
+      <c r="S17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T17" s="1"/>
-      <c r="V17" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T17" s="1">
+        <v>90</v>
+      </c>
+      <c r="V17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W17" s="1"/>
-      <c r="Y17" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W17" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z17" s="1"/>
-      <c r="AB17" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Z17" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17,$AC17), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC17" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="AC17" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
@@ -2210,14 +2228,14 @@
       </c>
       <c r="E27" s="10">
         <f>SUM(D14:D24)</f>
-        <v>5</v>
+        <v>-15</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H27" s="10">
         <f>SUM(G14:G24)</f>
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>7</v>
@@ -2231,35 +2249,35 @@
       </c>
       <c r="N27" s="10">
         <f>SUM(M14:M24)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q27" s="10">
         <f>SUM(P14:P24)</f>
-        <v>-30</v>
+        <v>-35</v>
       </c>
       <c r="S27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T27" s="10">
         <f>SUM(S14:S24)</f>
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="V27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W27" s="10">
         <f>SUM(V14:V24)</f>
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="Y27" s="26" t="s">
         <v>7</v>
       </c>
       <c r="Z27" s="10">
         <f>SUM(Y14:Y24)</f>
-        <v>-20</v>
+        <v>-45</v>
       </c>
       <c r="AA27" s="25"/>
       <c r="AB27" s="26" t="s">
@@ -2267,7 +2285,7 @@
       </c>
       <c r="AC27" s="10">
         <f>SUM(AB14:AB24)</f>
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AD27" s="1">
         <f>SUM(E27,H27,K27,N27,Q27,T27,W27,Z27,AC27)</f>

</xml_diff>

<commit_message>
Contest 5: GT vs PBKS
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{069CB805-D01F-8F40-A854-389F6F17706D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694550E7-05DE-9C42-8D00-3C01177A1B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -437,7 +437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -475,9 +475,7 @@
     <xf numFmtId="2" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -487,8 +485,9 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
@@ -502,6 +501,166 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -632,166 +791,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1342,10 +1341,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="21"/>
+      <c r="E12" s="25"/>
       <c r="G12" s="22" t="s">
         <v>14</v>
       </c>
@@ -1750,51 +1749,69 @@
       <c r="C18" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="3" t="str">
+      <c r="D18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E18" s="1"/>
-      <c r="G18" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E18" s="1">
+        <v>90</v>
+      </c>
+      <c r="G18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H18" s="1"/>
-      <c r="J18" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H18" s="1">
+        <v>30</v>
+      </c>
+      <c r="J18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K18" s="1"/>
-      <c r="M18" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K18" s="1">
+        <v>100</v>
+      </c>
+      <c r="M18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N18" s="1"/>
-      <c r="P18" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N18" s="1">
+        <v>40</v>
+      </c>
+      <c r="P18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q18" s="1"/>
-      <c r="S18" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>80</v>
+      </c>
+      <c r="S18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T18" s="1"/>
-      <c r="V18" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T18" s="1">
+        <v>50</v>
+      </c>
+      <c r="V18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W18" s="1"/>
-      <c r="Y18" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z18" s="1"/>
-      <c r="AB18" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="1">
+        <v>70</v>
+      </c>
+      <c r="AB18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18,$AC18), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC18" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="AC18" s="1">
+        <v>60</v>
+      </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
@@ -2228,64 +2245,63 @@
       </c>
       <c r="E27" s="10">
         <f>SUM(D14:D24)</f>
-        <v>-15</v>
+        <v>5</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H27" s="10">
         <f>SUM(G14:G24)</f>
-        <v>-5</v>
+        <v>-25</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K27" s="10">
         <f>SUM(J14:J24)</f>
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N27" s="10">
         <f>SUM(M14:M24)</f>
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="P27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q27" s="10">
         <f>SUM(P14:P24)</f>
-        <v>-35</v>
+        <v>-30</v>
       </c>
       <c r="S27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T27" s="10">
         <f>SUM(S14:S24)</f>
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="V27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W27" s="10">
         <f>SUM(V14:V24)</f>
-        <v>65</v>
-      </c>
-      <c r="Y27" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y27" s="21" t="s">
         <v>7</v>
       </c>
       <c r="Z27" s="10">
         <f>SUM(Y14:Y24)</f>
         <v>-45</v>
       </c>
-      <c r="AA27" s="25"/>
-      <c r="AB27" s="26" t="s">
+      <c r="AB27" s="21" t="s">
         <v>7</v>
       </c>
       <c r="AC27" s="10">
         <f>SUM(AB14:AB24)</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="AD27" s="1">
         <f>SUM(E27,H27,K27,N27,Q27,T27,W27,Z27,AC27)</f>
@@ -2295,66 +2311,66 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
   </mergeCells>
   <conditionalFormatting sqref="E27">
-    <cfRule type="cellIs" dxfId="29" priority="148" operator="lessThan">
+    <cfRule type="cellIs" dxfId="29" priority="150" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="28" priority="149" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="150" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="148" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H27">
-    <cfRule type="cellIs" dxfId="26" priority="43" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="45" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="44" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="45" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="43" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K27">
-    <cfRule type="cellIs" dxfId="23" priority="40" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="42" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="41" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="42" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="40" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N27">
-    <cfRule type="cellIs" dxfId="20" priority="37" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="39" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="38" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="37" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q27">
-    <cfRule type="cellIs" dxfId="17" priority="34" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="35" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="34" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="15" priority="36" operator="greaterThan">
@@ -2362,46 +2378,46 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T27">
-    <cfRule type="cellIs" dxfId="14" priority="31" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="33" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="13" priority="32" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="33" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="31" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W27">
-    <cfRule type="cellIs" dxfId="11" priority="28" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="30" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="29" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="30" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="28" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z27">
-    <cfRule type="cellIs" dxfId="8" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC27">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3101,13 +3117,13 @@
     <sortCondition descending="1" ref="K69:K77"/>
   </sortState>
   <conditionalFormatting sqref="K69:K77">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
13	1	LSG vs PBKS
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE2D8E5-6C89-8D40-AB5C-3F0603A34B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B26029-C311-A54A-B2C1-6B8B6E7499AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -510,8 +510,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -519,255 +519,15 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="54">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="30">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1415,24 +1175,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="26"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1441,22 +1201,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26"/>
-      <c r="T3" s="26"/>
-      <c r="U3" s="26"/>
-      <c r="V3" s="26"/>
-      <c r="W3" s="26"/>
-      <c r="X3" s="26"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1465,22 +1225,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="26"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="26"/>
-      <c r="T4" s="26"/>
-      <c r="U4" s="26"/>
-      <c r="V4" s="26"/>
-      <c r="W4" s="26"/>
-      <c r="X4" s="26"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1489,22 +1249,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-      <c r="Q5" s="26"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="26"/>
-      <c r="T5" s="26"/>
-      <c r="U5" s="26"/>
-      <c r="V5" s="26"/>
-      <c r="W5" s="26"/>
-      <c r="X5" s="26"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
+      <c r="R5" s="23"/>
+      <c r="S5" s="23"/>
+      <c r="T5" s="23"/>
+      <c r="U5" s="23"/>
+      <c r="V5" s="23"/>
+      <c r="W5" s="23"/>
+      <c r="X5" s="23"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1513,22 +1273,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="26"/>
-      <c r="T6" s="26"/>
-      <c r="U6" s="26"/>
-      <c r="V6" s="26"/>
-      <c r="W6" s="26"/>
-      <c r="X6" s="26"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="23"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="23"/>
+      <c r="X6" s="23"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1537,22 +1297,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="26"/>
-      <c r="O7" s="26"/>
-      <c r="P7" s="26"/>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="26"/>
-      <c r="S7" s="26"/>
-      <c r="T7" s="26"/>
-      <c r="U7" s="26"/>
-      <c r="V7" s="26"/>
-      <c r="W7" s="26"/>
-      <c r="X7" s="26"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="23"/>
+      <c r="R7" s="23"/>
+      <c r="S7" s="23"/>
+      <c r="T7" s="23"/>
+      <c r="U7" s="23"/>
+      <c r="V7" s="23"/>
+      <c r="W7" s="23"/>
+      <c r="X7" s="23"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1561,22 +1321,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="M8" s="26"/>
-      <c r="N8" s="26"/>
-      <c r="O8" s="26"/>
-      <c r="P8" s="26"/>
-      <c r="Q8" s="26"/>
-      <c r="R8" s="26"/>
-      <c r="S8" s="26"/>
-      <c r="T8" s="26"/>
-      <c r="U8" s="26"/>
-      <c r="V8" s="26"/>
-      <c r="W8" s="26"/>
-      <c r="X8" s="26"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="23"/>
+      <c r="R8" s="23"/>
+      <c r="S8" s="23"/>
+      <c r="T8" s="23"/>
+      <c r="U8" s="23"/>
+      <c r="V8" s="23"/>
+      <c r="W8" s="23"/>
+      <c r="X8" s="23"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1585,22 +1345,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="26"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="26"/>
-      <c r="P9" s="26"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="26"/>
-      <c r="T9" s="26"/>
-      <c r="U9" s="26"/>
-      <c r="V9" s="26"/>
-      <c r="W9" s="26"/>
-      <c r="X9" s="26"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="23"/>
+      <c r="R9" s="23"/>
+      <c r="S9" s="23"/>
+      <c r="T9" s="23"/>
+      <c r="U9" s="23"/>
+      <c r="V9" s="23"/>
+      <c r="W9" s="23"/>
+      <c r="X9" s="23"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1615,10 +1375,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="23"/>
+      <c r="E12" s="26"/>
       <c r="G12" s="24" t="s">
         <v>14</v>
       </c>
@@ -2613,51 +2373,67 @@
       <c r="C26" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="3" t="str">
+      <c r="D26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="G26" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H26" s="4"/>
-      <c r="J26" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K26" s="4"/>
-      <c r="M26" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0</v>
+      </c>
+      <c r="G26" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="H26" s="4">
+        <v>60</v>
+      </c>
+      <c r="J26" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="K26" s="4">
+        <v>60</v>
+      </c>
+      <c r="M26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N26" s="4"/>
-      <c r="P26" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N26" s="4">
+        <v>100</v>
+      </c>
+      <c r="P26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q26" s="4"/>
-      <c r="S26" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="4">
+        <v>70</v>
+      </c>
+      <c r="S26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T26" s="4"/>
-      <c r="V26" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T26" s="4">
+        <v>30</v>
+      </c>
+      <c r="V26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W26" s="4"/>
-      <c r="Y26" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W26" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z26" s="4"/>
-      <c r="AB26" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Z26" s="4">
+        <v>40</v>
+      </c>
+      <c r="AB26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26,$AC26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC26" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="AC26" s="4">
+        <v>80</v>
+      </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
@@ -3259,28 +3035,28 @@
       </c>
       <c r="E38" s="10">
         <f>SUM(D14:D35)</f>
-        <v>-10</v>
+        <v>-35</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-20</v>
+        <v>-27.5</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K38" s="10">
         <f>SUM(J14:J35)</f>
-        <v>5</v>
+        <v>-2.5</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N38" s="10">
         <f>SUM(M14:M35)</f>
-        <v>62.5</v>
+        <v>112.5</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>7</v>
@@ -3294,28 +3070,28 @@
       </c>
       <c r="T38" s="10">
         <f>SUM(S14:S35)</f>
-        <v>-25</v>
+        <v>-45</v>
       </c>
       <c r="V38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W38" s="10">
         <f>SUM(V14:V35)</f>
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="Y38" s="21" t="s">
         <v>7</v>
       </c>
       <c r="Z38" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-92.5</v>
+        <v>-107.5</v>
       </c>
       <c r="AB38" s="21" t="s">
         <v>7</v>
       </c>
       <c r="AC38" s="10">
         <f>SUM(AB14:AB35)</f>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="AD38" s="1">
         <f>SUM(E38,H38,K38,N38,Q38,T38,W38,Z38,AC38)</f>
@@ -3325,113 +3101,113 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
   <conditionalFormatting sqref="E38">
-    <cfRule type="cellIs" dxfId="53" priority="174" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="174" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="173" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="173" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="172" operator="lessThan">
+    <cfRule type="cellIs" dxfId="27" priority="172" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38">
-    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K38">
-    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N38">
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q38">
-    <cfRule type="cellIs" dxfId="12" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T38">
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W38">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z38">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC38">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4131,13 +3907,13 @@
     <sortCondition descending="1" ref="K69:K77"/>
   </sortState>
   <conditionalFormatting sqref="K69:K77">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
14 RCB vs GT
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B26029-C311-A54A-B2C1-6B8B6E7499AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01EE691A-5D4D-714C-921B-6536DC349F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -510,8 +510,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -519,8 +519,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1175,24 +1175,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="26"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1201,22 +1201,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="23"/>
-      <c r="Q3" s="23"/>
-      <c r="R3" s="23"/>
-      <c r="S3" s="23"/>
-      <c r="T3" s="23"/>
-      <c r="U3" s="23"/>
-      <c r="V3" s="23"/>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1225,22 +1225,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="23"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="26"/>
+      <c r="T4" s="26"/>
+      <c r="U4" s="26"/>
+      <c r="V4" s="26"/>
+      <c r="W4" s="26"/>
+      <c r="X4" s="26"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1249,22 +1249,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
-      <c r="T5" s="23"/>
-      <c r="U5" s="23"/>
-      <c r="V5" s="23"/>
-      <c r="W5" s="23"/>
-      <c r="X5" s="23"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="26"/>
+      <c r="R5" s="26"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="26"/>
+      <c r="W5" s="26"/>
+      <c r="X5" s="26"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1273,22 +1273,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="23"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="23"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="23"/>
-      <c r="X6" s="23"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="26"/>
+      <c r="T6" s="26"/>
+      <c r="U6" s="26"/>
+      <c r="V6" s="26"/>
+      <c r="W6" s="26"/>
+      <c r="X6" s="26"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1297,22 +1297,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="23"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="23"/>
-      <c r="T7" s="23"/>
-      <c r="U7" s="23"/>
-      <c r="V7" s="23"/>
-      <c r="W7" s="23"/>
-      <c r="X7" s="23"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1321,22 +1321,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="23"/>
-      <c r="Q8" s="23"/>
-      <c r="R8" s="23"/>
-      <c r="S8" s="23"/>
-      <c r="T8" s="23"/>
-      <c r="U8" s="23"/>
-      <c r="V8" s="23"/>
-      <c r="W8" s="23"/>
-      <c r="X8" s="23"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
+      <c r="N8" s="26"/>
+      <c r="O8" s="26"/>
+      <c r="P8" s="26"/>
+      <c r="Q8" s="26"/>
+      <c r="R8" s="26"/>
+      <c r="S8" s="26"/>
+      <c r="T8" s="26"/>
+      <c r="U8" s="26"/>
+      <c r="V8" s="26"/>
+      <c r="W8" s="26"/>
+      <c r="X8" s="26"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1345,22 +1345,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="23"/>
-      <c r="S9" s="23"/>
-      <c r="T9" s="23"/>
-      <c r="U9" s="23"/>
-      <c r="V9" s="23"/>
-      <c r="W9" s="23"/>
-      <c r="X9" s="23"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="26"/>
+      <c r="S9" s="26"/>
+      <c r="T9" s="26"/>
+      <c r="U9" s="26"/>
+      <c r="V9" s="26"/>
+      <c r="W9" s="26"/>
+      <c r="X9" s="26"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1375,10 +1375,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="26"/>
+      <c r="E12" s="23"/>
       <c r="G12" s="24" t="s">
         <v>14</v>
       </c>
@@ -2445,51 +2445,69 @@
       <c r="C27" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="3" t="str">
+      <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="G27" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E27" s="4">
+        <v>100</v>
+      </c>
+      <c r="G27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H27" s="4"/>
-      <c r="J27" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H27" s="4">
+        <v>60</v>
+      </c>
+      <c r="J27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K27" s="4"/>
-      <c r="M27" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K27" s="4">
+        <v>40</v>
+      </c>
+      <c r="M27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N27" s="4"/>
-      <c r="P27" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N27" s="4">
+        <v>0</v>
+      </c>
+      <c r="P27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q27" s="4"/>
-      <c r="S27" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q27" s="4">
+        <v>80</v>
+      </c>
+      <c r="S27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T27" s="4"/>
-      <c r="V27" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T27" s="4">
+        <v>30</v>
+      </c>
+      <c r="V27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W27" s="4"/>
-      <c r="Y27" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W27" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z27" s="4"/>
-      <c r="AB27" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Z27" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27,$AC27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC27" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC27" s="4">
+        <v>70</v>
+      </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
@@ -3035,56 +3053,56 @@
       </c>
       <c r="E38" s="10">
         <f>SUM(D14:D35)</f>
-        <v>-35</v>
+        <v>15</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-27.5</v>
+        <v>-32.5</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K38" s="10">
         <f>SUM(J14:J35)</f>
-        <v>-2.5</v>
+        <v>-17.5</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N38" s="10">
         <f>SUM(M14:M35)</f>
-        <v>112.5</v>
+        <v>87.5</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q38" s="10">
         <f>SUM(P14:P35)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="S38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T38" s="10">
         <f>SUM(S14:S35)</f>
-        <v>-45</v>
+        <v>-65</v>
       </c>
       <c r="V38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W38" s="10">
         <f>SUM(V14:V35)</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="Y38" s="21" t="s">
         <v>7</v>
       </c>
       <c r="Z38" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-107.5</v>
+        <v>-117.5</v>
       </c>
       <c r="AB38" s="21" t="s">
         <v>7</v>
@@ -3101,16 +3119,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E38">
     <cfRule type="cellIs" dxfId="29" priority="174" operator="greaterThan">

</xml_diff>

<commit_message>
15	1	KKR vs SRH
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5777479A-E211-3341-A680-E8E774B24334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7948703-ADEF-CE41-B408-3771E9AE510C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" activeTab="1" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -417,8 +417,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -426,45 +426,15 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1082,24 +1052,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1108,22 +1078,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1132,22 +1102,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1156,22 +1126,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1180,22 +1150,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1204,22 +1174,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1228,22 +1198,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1252,22 +1222,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1282,10 +1252,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="22"/>
+      <c r="E12" s="19"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -2426,51 +2396,69 @@
       <c r="C28" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D28" s="3" t="str">
+      <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E28" s="4"/>
-      <c r="G28" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E28" s="4">
+        <v>0</v>
+      </c>
+      <c r="G28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H28" s="4"/>
-      <c r="J28" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H28" s="4">
+        <v>80</v>
+      </c>
+      <c r="J28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K28" s="4"/>
-      <c r="M28" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="K28" s="4">
+        <v>70</v>
+      </c>
+      <c r="M28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N28" s="4"/>
-      <c r="P28" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N28" s="4">
+        <v>90</v>
+      </c>
+      <c r="P28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q28" s="4"/>
-      <c r="S28" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q28" s="4">
+        <v>30</v>
+      </c>
+      <c r="S28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T28" s="4"/>
-      <c r="V28" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T28" s="4">
+        <v>50</v>
+      </c>
+      <c r="V28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W28" s="4"/>
-      <c r="Y28" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W28" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z28" s="4"/>
-      <c r="AB28" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Z28" s="4">
+        <v>60</v>
+      </c>
+      <c r="AB28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28,$AC28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC28" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="AC28" s="4">
+        <v>100</v>
+      </c>
     </row>
     <row r="29" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
@@ -2960,14 +2948,14 @@
       </c>
       <c r="E38" s="10">
         <f>SUM(D14:D35)</f>
-        <v>15</v>
+        <v>-10</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-32.5</v>
+        <v>-27.5</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>7</v>
@@ -2981,42 +2969,42 @@
       </c>
       <c r="N38" s="10">
         <f>SUM(M14:M35)</f>
-        <v>87.5</v>
+        <v>107.5</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q38" s="10">
         <f>SUM(P14:P35)</f>
-        <v>10</v>
+        <v>-10</v>
       </c>
       <c r="S38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T38" s="10">
         <f>SUM(S14:S35)</f>
-        <v>-65</v>
+        <v>-75</v>
       </c>
       <c r="V38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W38" s="10">
         <f>SUM(V14:V35)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="Y38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z38" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-117.5</v>
+        <v>-122.5</v>
       </c>
       <c r="AB38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC38" s="10">
         <f>SUM(AB14:AB35)</f>
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="AD38" s="1">
         <f>SUM(E38,H38,K38,N38,Q38,T38,W38,Z38,AC38)</f>
@@ -3026,113 +3014,113 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E38">
-    <cfRule type="cellIs" dxfId="29" priority="174" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="174" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="173" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="173" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="172" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="172" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38">
-    <cfRule type="cellIs" dxfId="26" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K38">
-    <cfRule type="cellIs" dxfId="23" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N38">
-    <cfRule type="cellIs" dxfId="20" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q38">
-    <cfRule type="cellIs" dxfId="17" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T38">
-    <cfRule type="cellIs" dxfId="14" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W38">
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z38">
-    <cfRule type="cellIs" dxfId="8" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC38">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
16, 17, 18 & 19
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7948703-ADEF-CE41-B408-3771E9AE510C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238280F4-6391-3C43-A00D-FF368A5283E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -417,8 +417,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -426,8 +426,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1052,24 +1052,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1078,22 +1078,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1102,22 +1102,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1126,22 +1126,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1150,22 +1150,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1174,22 +1174,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1198,22 +1198,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1222,22 +1222,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1252,10 +1252,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="19"/>
+      <c r="E12" s="22"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -2470,51 +2470,69 @@
       <c r="C29" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="D29" s="3" t="str">
+      <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="G29" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E29" s="4">
+        <v>100</v>
+      </c>
+      <c r="G29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H29" s="4"/>
-      <c r="J29" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4">
+        <v>70</v>
+      </c>
+      <c r="J29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K29" s="4"/>
-      <c r="M29" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K29" s="4">
+        <v>40</v>
+      </c>
+      <c r="M29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N29" s="4"/>
-      <c r="P29" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N29" s="4">
+        <v>90</v>
+      </c>
+      <c r="P29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q29" s="4"/>
-      <c r="S29" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q29" s="4">
+        <v>30</v>
+      </c>
+      <c r="S29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T29" s="4"/>
-      <c r="V29" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T29" s="4">
+        <v>80</v>
+      </c>
+      <c r="V29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W29" s="4"/>
-      <c r="Y29" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W29" s="4">
+        <v>50</v>
+      </c>
+      <c r="Y29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z29" s="4"/>
-      <c r="AB29" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Z29" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29,$AC29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC29" s="4"/>
+        <v>-5</v>
+      </c>
+      <c r="AC29" s="4">
+        <v>60</v>
+      </c>
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
@@ -2526,51 +2544,69 @@
       <c r="C30" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="D30" s="3" t="str">
+      <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E30" s="4"/>
-      <c r="G30" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E30" s="4">
+        <v>60</v>
+      </c>
+      <c r="G30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H30" s="4"/>
-      <c r="J30" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H30" s="4">
+        <v>30</v>
+      </c>
+      <c r="J30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K30" s="4"/>
-      <c r="M30" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K30" s="4">
+        <v>100</v>
+      </c>
+      <c r="M30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N30" s="4"/>
-      <c r="P30" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N30" s="4">
+        <v>50</v>
+      </c>
+      <c r="P30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q30" s="4"/>
-      <c r="S30" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q30" s="4">
+        <v>90</v>
+      </c>
+      <c r="S30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T30" s="4"/>
-      <c r="V30" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T30" s="4">
+        <v>40</v>
+      </c>
+      <c r="V30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W30" s="4"/>
-      <c r="Y30" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="W30" s="4">
+        <v>70</v>
+      </c>
+      <c r="Y30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z30" s="4"/>
-      <c r="AB30" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Z30" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30,$AC30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC30" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="AC30" s="4">
+        <v>80</v>
+      </c>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
@@ -2582,51 +2618,67 @@
       <c r="C31" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="3" t="str">
+      <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E31" s="4"/>
-      <c r="G31" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H31" s="4"/>
-      <c r="J31" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E31" s="4">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="H31" s="4">
+        <v>60</v>
+      </c>
+      <c r="J31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K31" s="4"/>
-      <c r="M31" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N31" s="4"/>
-      <c r="P31" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K31" s="4">
+        <v>90</v>
+      </c>
+      <c r="M31" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="N31" s="4">
+        <v>60</v>
+      </c>
+      <c r="P31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q31" s="4"/>
-      <c r="S31" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q31" s="4">
+        <v>30</v>
+      </c>
+      <c r="S31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T31" s="4"/>
-      <c r="V31" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T31" s="4">
+        <v>100</v>
+      </c>
+      <c r="V31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W31" s="4"/>
-      <c r="Y31" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W31" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z31" s="4"/>
-      <c r="AB31" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z31" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31,$AC31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC31" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC31" s="4">
+        <v>70</v>
+      </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
@@ -2638,51 +2690,67 @@
       <c r="C32" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="3" t="str">
+      <c r="D32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E32" s="4"/>
-      <c r="G32" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E32" s="4">
+        <v>100</v>
+      </c>
+      <c r="G32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H32" s="4"/>
-      <c r="J32" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H32" s="4">
+        <v>50</v>
+      </c>
+      <c r="J32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K32" s="4"/>
-      <c r="M32" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K32" s="4">
+        <v>60</v>
+      </c>
+      <c r="M32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N32" s="4"/>
-      <c r="P32" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N32" s="4">
+        <v>30</v>
+      </c>
+      <c r="P32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q32" s="4"/>
-      <c r="S32" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q32" s="4">
+        <v>40</v>
+      </c>
+      <c r="S32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T32" s="4"/>
-      <c r="V32" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T32" s="4">
+        <v>90</v>
+      </c>
+      <c r="V32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W32" s="4"/>
-      <c r="Y32" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z32" s="4"/>
-      <c r="AB32" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(AC32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32,$AC32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC32" s="4"/>
+        <v>-25</v>
+      </c>
+      <c r="W32" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="Z32" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB32" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="AC32" s="4">
+        <v>80</v>
+      </c>
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
@@ -2948,63 +3016,63 @@
       </c>
       <c r="E38" s="10">
         <f>SUM(D14:D35)</f>
-        <v>-10</v>
+        <v>60</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-27.5</v>
+        <v>-65</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K38" s="10">
         <f>SUM(J14:J35)</f>
-        <v>-17.5</v>
+        <v>32.5</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N38" s="10">
         <f>SUM(M14:M35)</f>
-        <v>107.5</v>
+        <v>90</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q38" s="10">
         <f>SUM(P14:P35)</f>
-        <v>-10</v>
+        <v>-45</v>
       </c>
       <c r="S38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T38" s="10">
         <f>SUM(S14:S35)</f>
-        <v>-75</v>
+        <v>-15</v>
       </c>
       <c r="V38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W38" s="10">
         <f>SUM(V14:V35)</f>
-        <v>15</v>
+        <v>-35</v>
       </c>
       <c r="Y38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z38" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-122.5</v>
+        <v>-165</v>
       </c>
       <c r="AB38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC38" s="10">
         <f>SUM(AB14:AB35)</f>
-        <v>140</v>
+        <v>142.5</v>
       </c>
       <c r="AD38" s="1">
         <f>SUM(E38,H38,K38,N38,Q38,T38,W38,Z38,AC38)</f>
@@ -3014,16 +3082,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
   <conditionalFormatting sqref="E38">
     <cfRule type="cellIs" dxfId="26" priority="174" operator="greaterThan">

</xml_diff>

<commit_message>
20	1	MI vs RCB
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238280F4-6391-3C43-A00D-FF368A5283E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7359C7-6AEA-BD49-990A-5F292644DDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -417,8 +417,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -426,8 +426,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1052,24 +1052,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1078,22 +1078,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1102,22 +1102,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1126,22 +1126,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1150,22 +1150,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1174,22 +1174,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1198,22 +1198,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1222,22 +1222,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1252,10 +1252,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="22"/>
+      <c r="E12" s="19"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -2762,51 +2762,69 @@
       <c r="C33" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D33" s="3" t="str">
+      <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E33" s="4"/>
-      <c r="G33" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="E33" s="4">
+        <v>70</v>
+      </c>
+      <c r="G33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H33" s="4"/>
-      <c r="J33" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H33" s="4">
+        <v>80</v>
+      </c>
+      <c r="J33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K33" s="4"/>
-      <c r="M33" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K33" s="4">
+        <v>60</v>
+      </c>
+      <c r="M33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N33" s="4"/>
-      <c r="P33" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N33" s="4">
+        <v>0</v>
+      </c>
+      <c r="P33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q33" s="4"/>
-      <c r="S33" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q33" s="4">
+        <v>40</v>
+      </c>
+      <c r="S33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T33" s="4"/>
-      <c r="V33" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T33" s="4">
+        <v>100</v>
+      </c>
+      <c r="V33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W33" s="4"/>
-      <c r="Y33" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W33" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z33" s="4"/>
-      <c r="AB33" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Z33" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33,$AC33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC33" s="4"/>
+        <v>-20</v>
+      </c>
+      <c r="AC33" s="4">
+        <v>30</v>
+      </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
@@ -3023,56 +3041,56 @@
       </c>
       <c r="H38" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-65</v>
+        <v>-60</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K38" s="10">
         <f>SUM(J14:J35)</f>
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N38" s="10">
         <f>SUM(M14:M35)</f>
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q38" s="10">
         <f>SUM(P14:P35)</f>
-        <v>-45</v>
+        <v>-60</v>
       </c>
       <c r="S38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T38" s="10">
         <f>SUM(S14:S35)</f>
-        <v>-15</v>
+        <v>35</v>
       </c>
       <c r="V38" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W38" s="10">
         <f>SUM(V14:V35)</f>
-        <v>-35</v>
+        <v>-15</v>
       </c>
       <c r="Y38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z38" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-165</v>
+        <v>-175</v>
       </c>
       <c r="AB38" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC38" s="10">
         <f>SUM(AB14:AB35)</f>
-        <v>142.5</v>
+        <v>122.5</v>
       </c>
       <c r="AD38" s="1">
         <f>SUM(E38,H38,K38,N38,Q38,T38,W38,Z38,AC38)</f>
@@ -3082,16 +3100,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E38">
     <cfRule type="cellIs" dxfId="26" priority="174" operator="greaterThan">

</xml_diff>

<commit_message>
contest 20 & 21
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7359C7-6AEA-BD49-990A-5F292644DDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A55B9E4-A18F-6847-84D1-C7F0FC67B558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="75">
   <si>
     <t>Points</t>
   </si>
@@ -219,6 +219,54 @@
   </si>
   <si>
     <t>PBKS vs CSK</t>
+  </si>
+  <si>
+    <t>GT vs RR</t>
+  </si>
+  <si>
+    <t>RCB vs DC</t>
+  </si>
+  <si>
+    <t>CSK vs KKR</t>
+  </si>
+  <si>
+    <t>LSG vs GT</t>
+  </si>
+  <si>
+    <t>SRH vs PBKS</t>
+  </si>
+  <si>
+    <t>RR vs RCB</t>
+  </si>
+  <si>
+    <t>DC vs MI</t>
+  </si>
+  <si>
+    <t>LSG vs CSK</t>
+  </si>
+  <si>
+    <t>PBKS vs KKR</t>
+  </si>
+  <si>
+    <t>DC vs RR</t>
+  </si>
+  <si>
+    <t>MI vs SRH</t>
+  </si>
+  <si>
+    <t>RCB vs PBKS</t>
+  </si>
+  <si>
+    <t>GT vs DC</t>
+  </si>
+  <si>
+    <t>RR vs LSG</t>
+  </si>
+  <si>
+    <t>PBKS vs RCB</t>
+  </si>
+  <si>
+    <t>MI vs CSK</t>
   </si>
 </sst>
 </file>
@@ -417,8 +465,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -426,8 +474,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -437,141 +485,11 @@
   <dxfs count="27">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -702,6 +620,136 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1020,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE9CB7-B9A7-B347-86F0-C3EB9B5BFBBD}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
@@ -1052,24 +1100,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1078,22 +1126,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1102,22 +1150,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1126,22 +1174,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1150,22 +1198,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1174,22 +1222,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1198,22 +1246,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1222,22 +1270,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1252,10 +1300,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="19"/>
+      <c r="E12" s="22"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -2752,7 +2800,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>20</v>
       </c>
@@ -2826,7 +2874,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>21</v>
       </c>
@@ -2836,53 +2884,71 @@
       <c r="C34" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D34" s="3" t="str">
+      <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E34" s="4"/>
-      <c r="G34" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="E34" s="4">
+        <v>30</v>
+      </c>
+      <c r="G34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H34" s="4"/>
-      <c r="J34" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H34" s="4">
+        <v>60</v>
+      </c>
+      <c r="J34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K34" s="4"/>
-      <c r="M34" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K34" s="4">
+        <v>100</v>
+      </c>
+      <c r="M34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N34" s="4"/>
-      <c r="P34" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N34" s="4">
+        <v>40</v>
+      </c>
+      <c r="P34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q34" s="4"/>
-      <c r="S34" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q34" s="4">
+        <v>50</v>
+      </c>
+      <c r="S34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T34" s="4"/>
-      <c r="V34" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="T34" s="4">
+        <v>70</v>
+      </c>
+      <c r="V34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W34" s="4"/>
-      <c r="Y34" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W34" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z34" s="4"/>
-      <c r="AB34" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Z34" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34,$AC34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC34" s="4"/>
-    </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="AC34" s="4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
         <v>22</v>
       </c>
@@ -2892,321 +2958,1233 @@
       <c r="C35" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D35" s="3" t="str">
+      <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E35" s="4"/>
-      <c r="G35" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E35" s="4">
+        <v>60</v>
+      </c>
+      <c r="G35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H35" s="4"/>
-      <c r="J35" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K35" s="4"/>
-      <c r="M35" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H35" s="4">
+        <v>30</v>
+      </c>
+      <c r="J35" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="K35" s="4">
+        <v>80</v>
+      </c>
+      <c r="M35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N35" s="4"/>
-      <c r="P35" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N35" s="4">
+        <v>40</v>
+      </c>
+      <c r="P35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q35" s="4"/>
-      <c r="S35" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q35" s="4">
+        <v>100</v>
+      </c>
+      <c r="S35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T35" s="4"/>
-      <c r="V35" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W35" s="4"/>
-      <c r="Y35" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T35" s="4">
+        <v>90</v>
+      </c>
+      <c r="V35" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="W35" s="4">
+        <v>80</v>
+      </c>
+      <c r="Y35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z35" s="4"/>
-      <c r="AB35" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Z35" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35,$AC35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC35" s="4"/>
-    </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A36" s="5"/>
-      <c r="B36" s="1" t="s">
+        <v>-10</v>
+      </c>
+      <c r="AC35" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>23</v>
+      </c>
+      <c r="B36" s="4">
+        <v>1</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E36" s="4"/>
+      <c r="G36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H36" s="4"/>
+      <c r="J36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K36" s="4"/>
+      <c r="M36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N36" s="4"/>
+      <c r="P36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q36" s="4"/>
+      <c r="S36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T36" s="4"/>
+      <c r="V36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W36" s="4"/>
+      <c r="Y36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z36" s="4"/>
+      <c r="AB36" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC36" s="4"/>
+    </row>
+    <row r="37" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A37" s="5">
+        <v>24</v>
+      </c>
+      <c r="B37" s="4">
+        <v>1</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E37" s="4"/>
+      <c r="G37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H37" s="4"/>
+      <c r="J37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K37" s="4"/>
+      <c r="M37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N37" s="4"/>
+      <c r="P37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q37" s="4"/>
+      <c r="S37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T37" s="4"/>
+      <c r="V37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W37" s="4"/>
+      <c r="Y37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z37" s="4"/>
+      <c r="AB37" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC37" s="4"/>
+    </row>
+    <row r="38" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>25</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E38" s="4"/>
+      <c r="G38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H38" s="4"/>
+      <c r="J38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K38" s="4"/>
+      <c r="M38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N38" s="4"/>
+      <c r="P38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q38" s="4"/>
+      <c r="S38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T38" s="4"/>
+      <c r="V38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W38" s="4"/>
+      <c r="Y38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z38" s="4"/>
+      <c r="AB38" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC38" s="4"/>
+    </row>
+    <row r="39" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A39" s="5">
+        <v>26</v>
+      </c>
+      <c r="B39" s="4">
+        <v>1</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E39" s="4"/>
+      <c r="G39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H39" s="4"/>
+      <c r="J39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K39" s="4"/>
+      <c r="M39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N39" s="4"/>
+      <c r="P39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q39" s="4"/>
+      <c r="S39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T39" s="4"/>
+      <c r="V39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W39" s="4"/>
+      <c r="Y39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z39" s="4"/>
+      <c r="AB39" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC39" s="4"/>
+    </row>
+    <row r="40" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>27</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E40" s="4"/>
+      <c r="G40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H40" s="4"/>
+      <c r="J40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K40" s="4"/>
+      <c r="M40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N40" s="4"/>
+      <c r="P40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q40" s="4"/>
+      <c r="S40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T40" s="4"/>
+      <c r="V40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W40" s="4"/>
+      <c r="Y40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z40" s="4"/>
+      <c r="AB40" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC40" s="4"/>
+    </row>
+    <row r="41" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A41" s="5">
+        <v>28</v>
+      </c>
+      <c r="B41" s="4">
+        <v>1</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E41" s="4"/>
+      <c r="G41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H41" s="4"/>
+      <c r="J41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K41" s="4"/>
+      <c r="M41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N41" s="4"/>
+      <c r="P41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q41" s="4"/>
+      <c r="S41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T41" s="4"/>
+      <c r="V41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W41" s="4"/>
+      <c r="Y41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z41" s="4"/>
+      <c r="AB41" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC41" s="4"/>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>29</v>
+      </c>
+      <c r="B42" s="4">
+        <v>1</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E42" s="4"/>
+      <c r="G42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H42" s="4"/>
+      <c r="J42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K42" s="4"/>
+      <c r="M42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N42" s="4"/>
+      <c r="P42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q42" s="4"/>
+      <c r="S42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T42" s="4"/>
+      <c r="V42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W42" s="4"/>
+      <c r="Y42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z42" s="4"/>
+      <c r="AB42" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC42" s="4"/>
+    </row>
+    <row r="43" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A43" s="5">
+        <v>30</v>
+      </c>
+      <c r="B43" s="4">
+        <v>1</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E43" s="4"/>
+      <c r="G43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H43" s="4"/>
+      <c r="J43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K43" s="4"/>
+      <c r="M43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N43" s="4"/>
+      <c r="P43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q43" s="4"/>
+      <c r="S43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T43" s="4"/>
+      <c r="V43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W43" s="4"/>
+      <c r="Y43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z43" s="4"/>
+      <c r="AB43" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43,$AC43), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC43" s="4"/>
+    </row>
+    <row r="44" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>31</v>
+      </c>
+      <c r="B44" s="4">
+        <v>1</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E44" s="4"/>
+      <c r="G44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H44" s="4"/>
+      <c r="J44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K44" s="4"/>
+      <c r="M44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N44" s="4"/>
+      <c r="P44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q44" s="4"/>
+      <c r="S44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T44" s="4"/>
+      <c r="V44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W44" s="4"/>
+      <c r="Y44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z44" s="4"/>
+      <c r="AB44" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC44" s="4"/>
+    </row>
+    <row r="45" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A45" s="5">
+        <v>32</v>
+      </c>
+      <c r="B45" s="4">
+        <v>1</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E45" s="4"/>
+      <c r="G45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H45" s="4"/>
+      <c r="J45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K45" s="4"/>
+      <c r="M45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N45" s="4"/>
+      <c r="P45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q45" s="4"/>
+      <c r="S45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T45" s="4"/>
+      <c r="V45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W45" s="4"/>
+      <c r="Y45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z45" s="4"/>
+      <c r="AB45" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC45" s="4"/>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>33</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E46" s="4"/>
+      <c r="G46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H46" s="4"/>
+      <c r="J46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K46" s="4"/>
+      <c r="M46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N46" s="4"/>
+      <c r="P46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q46" s="4"/>
+      <c r="S46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T46" s="4"/>
+      <c r="V46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W46" s="4"/>
+      <c r="Y46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z46" s="4"/>
+      <c r="AB46" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46,$AC46), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC46" s="4"/>
+    </row>
+    <row r="47" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A47" s="5">
+        <v>34</v>
+      </c>
+      <c r="B47" s="4">
+        <v>1</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E47" s="4"/>
+      <c r="G47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H47" s="4"/>
+      <c r="J47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K47" s="4"/>
+      <c r="M47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N47" s="4"/>
+      <c r="P47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q47" s="4"/>
+      <c r="S47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T47" s="4"/>
+      <c r="V47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W47" s="4"/>
+      <c r="Y47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z47" s="4"/>
+      <c r="AB47" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47,$AC47), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC47" s="4"/>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>35</v>
+      </c>
+      <c r="B48" s="4">
+        <v>1</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E48" s="4"/>
+      <c r="G48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H48" s="4"/>
+      <c r="J48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K48" s="4"/>
+      <c r="M48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N48" s="4"/>
+      <c r="P48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q48" s="4"/>
+      <c r="S48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T48" s="4"/>
+      <c r="V48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W48" s="4"/>
+      <c r="Y48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z48" s="4"/>
+      <c r="AB48" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48,$AC48), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC48" s="4"/>
+    </row>
+    <row r="49" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A49" s="5">
+        <v>36</v>
+      </c>
+      <c r="B49" s="4">
+        <v>1</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E49" s="4"/>
+      <c r="G49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H49" s="4"/>
+      <c r="J49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K49" s="4"/>
+      <c r="M49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N49" s="4"/>
+      <c r="P49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q49" s="4"/>
+      <c r="S49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T49" s="4"/>
+      <c r="V49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W49" s="4"/>
+      <c r="Y49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z49" s="4"/>
+      <c r="AB49" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49,$AC49), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC49" s="4"/>
+    </row>
+    <row r="50" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>37</v>
+      </c>
+      <c r="B50" s="4">
+        <v>1</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E50" s="4"/>
+      <c r="G50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H50" s="4"/>
+      <c r="J50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K50" s="4"/>
+      <c r="M50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N50" s="4"/>
+      <c r="P50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q50" s="4"/>
+      <c r="S50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T50" s="4"/>
+      <c r="V50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W50" s="4"/>
+      <c r="Y50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z50" s="4"/>
+      <c r="AB50" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50,$AC50), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC50" s="4"/>
+    </row>
+    <row r="51" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A51" s="5">
+        <v>38</v>
+      </c>
+      <c r="B51" s="4">
+        <v>1</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E51" s="4"/>
+      <c r="G51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H51" s="4"/>
+      <c r="J51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K51" s="4"/>
+      <c r="M51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N51" s="4"/>
+      <c r="P51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q51" s="4"/>
+      <c r="S51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T51" s="4"/>
+      <c r="V51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W51" s="4"/>
+      <c r="Y51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z51" s="4"/>
+      <c r="AB51" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51,$AC51), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC51" s="4"/>
+    </row>
+    <row r="52" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A52" s="5"/>
+      <c r="B52" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="7" t="s">
+      <c r="C52" s="8"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="7" t="s">
+      <c r="G52" s="1"/>
+      <c r="H52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="J36" s="1"/>
-      <c r="K36" s="7" t="s">
+      <c r="J52" s="1"/>
+      <c r="K52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="M36" s="1"/>
-      <c r="N36" s="7" t="s">
+      <c r="M52" s="1"/>
+      <c r="N52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="P36" s="1"/>
-      <c r="Q36" s="7" t="s">
+      <c r="P52" s="1"/>
+      <c r="Q52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="S36" s="1"/>
-      <c r="T36" s="7" t="s">
+      <c r="S52" s="1"/>
+      <c r="T52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="V36" s="1"/>
-      <c r="W36" s="7" t="s">
+      <c r="V52" s="1"/>
+      <c r="W52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="Y36" s="1"/>
-      <c r="Z36" s="7" t="s">
+      <c r="Y52" s="1"/>
+      <c r="Z52" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AB36" s="1"/>
-      <c r="AC36" s="7" t="s">
+      <c r="AB52" s="1"/>
+      <c r="AC52" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="D37" s="1"/>
-      <c r="E37" s="9" t="str">
+    <row r="53" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="D53" s="1"/>
+      <c r="E53" s="9" t="str">
         <f>D13</f>
         <v>Jaya</v>
       </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="9" t="str">
+      <c r="G53" s="1"/>
+      <c r="H53" s="9" t="str">
         <f>G13</f>
         <v>Justin</v>
       </c>
-      <c r="J37" s="1"/>
-      <c r="K37" s="9" t="str">
+      <c r="J53" s="1"/>
+      <c r="K53" s="9" t="str">
         <f>J13</f>
         <v>Ram</v>
       </c>
-      <c r="M37" s="1"/>
-      <c r="N37" s="9" t="str">
+      <c r="M53" s="1"/>
+      <c r="N53" s="9" t="str">
         <f>M13</f>
         <v>Sibi</v>
       </c>
-      <c r="P37" s="1"/>
-      <c r="Q37" s="9" t="str">
+      <c r="P53" s="1"/>
+      <c r="Q53" s="9" t="str">
         <f>P13</f>
         <v>Sundar</v>
       </c>
-      <c r="S37" s="1"/>
-      <c r="T37" s="9" t="str">
+      <c r="S53" s="1"/>
+      <c r="T53" s="9" t="str">
         <f>S13</f>
         <v>Sampath</v>
       </c>
-      <c r="V37" s="1"/>
-      <c r="W37" s="9" t="str">
+      <c r="V53" s="1"/>
+      <c r="W53" s="9" t="str">
         <f>V13</f>
         <v>Jayanth</v>
       </c>
-      <c r="Y37" s="1"/>
-      <c r="Z37" s="9" t="str">
+      <c r="Y53" s="1"/>
+      <c r="Z53" s="9" t="str">
         <f>Y13</f>
         <v>Vicky</v>
       </c>
-      <c r="AB37" s="1"/>
-      <c r="AC37" s="9" t="str">
+      <c r="AB53" s="1"/>
+      <c r="AC53" s="9" t="str">
         <f>AB13</f>
         <v>Anantha</v>
       </c>
     </row>
-    <row r="38" spans="1:30" ht="21" x14ac:dyDescent="0.25">
-      <c r="D38" s="6" t="s">
+    <row r="54" spans="1:30" ht="21" x14ac:dyDescent="0.25">
+      <c r="D54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E38" s="10">
+      <c r="E54" s="10">
         <f>SUM(D14:D35)</f>
-        <v>60</v>
-      </c>
-      <c r="G38" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H38" s="10">
+      <c r="H54" s="10">
         <f>SUM(G14:G35)</f>
-        <v>-60</v>
-      </c>
-      <c r="J38" s="6" t="s">
+        <v>-85</v>
+      </c>
+      <c r="J54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K38" s="10">
+      <c r="K54" s="10">
         <f>SUM(J14:J35)</f>
-        <v>27.5</v>
-      </c>
-      <c r="M38" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="N38" s="10">
+      <c r="N54" s="10">
         <f>SUM(M14:M35)</f>
-        <v>65</v>
-      </c>
-      <c r="P38" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="P54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="Q38" s="10">
+      <c r="Q54" s="10">
         <f>SUM(P14:P35)</f>
-        <v>-60</v>
-      </c>
-      <c r="S38" s="6" t="s">
+        <v>-20</v>
+      </c>
+      <c r="S54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="T38" s="10">
+      <c r="T54" s="10">
         <f>SUM(S14:S35)</f>
-        <v>35</v>
-      </c>
-      <c r="V38" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="W38" s="10">
+      <c r="W54" s="10">
         <f>SUM(V14:V35)</f>
-        <v>-15</v>
-      </c>
-      <c r="Y38" s="17" t="s">
+        <v>7.5</v>
+      </c>
+      <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Z38" s="10">
+      <c r="Z54" s="10">
         <f>SUM(Y14:Y35)</f>
-        <v>-175</v>
-      </c>
-      <c r="AB38" s="17" t="s">
+        <v>-225</v>
+      </c>
+      <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="AC38" s="10">
+      <c r="AC54" s="10">
         <f>SUM(AB14:AB35)</f>
-        <v>122.5</v>
-      </c>
-      <c r="AD38" s="1">
-        <f>SUM(E38,H38,K38,N38,Q38,T38,W38,Z38,AC38)</f>
+        <v>117.5</v>
+      </c>
+      <c r="AD54" s="1">
+        <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
-  <conditionalFormatting sqref="E38">
-    <cfRule type="cellIs" dxfId="26" priority="174" operator="greaterThan">
+  <conditionalFormatting sqref="E54">
+    <cfRule type="cellIs" dxfId="26" priority="172" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="173" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="172" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="174" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H38">
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
+  <conditionalFormatting sqref="H54">
+    <cfRule type="cellIs" dxfId="23" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K38">
-    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
+  <conditionalFormatting sqref="K54">
+    <cfRule type="cellIs" dxfId="20" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N38">
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
+  <conditionalFormatting sqref="N54">
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q38">
-    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+  <conditionalFormatting sqref="Q54">
+    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T38">
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
+  <conditionalFormatting sqref="T54">
+    <cfRule type="cellIs" dxfId="11" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W38">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
+  <conditionalFormatting sqref="W54">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z38">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+  <conditionalFormatting sqref="Z54">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC38">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+  <conditionalFormatting sqref="AC54">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
23 GT vs RR
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A55B9E4-A18F-6847-84D1-C7F0FC67B558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B67C5E-D9CE-C447-8552-B1CD54F1D4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -482,7 +482,247 @@
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="51">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -3030,51 +3270,69 @@
       <c r="C36" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="3" t="str">
+      <c r="D36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E36" s="4"/>
-      <c r="G36" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E36" s="4">
+        <v>80</v>
+      </c>
+      <c r="G36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H36" s="4"/>
-      <c r="J36" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H36" s="4">
+        <v>50</v>
+      </c>
+      <c r="J36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K36" s="4"/>
-      <c r="M36" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K36" s="4">
+        <v>60</v>
+      </c>
+      <c r="M36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N36" s="4"/>
-      <c r="P36" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N36" s="4">
+        <v>0</v>
+      </c>
+      <c r="P36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q36" s="4"/>
-      <c r="S36" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q36" s="4">
+        <v>90</v>
+      </c>
+      <c r="S36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T36" s="4"/>
-      <c r="V36" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T36" s="4">
+        <v>30</v>
+      </c>
+      <c r="V36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W36" s="4"/>
-      <c r="Y36" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W36" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z36" s="4"/>
-      <c r="AB36" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="4">
+        <v>70</v>
+      </c>
+      <c r="AB36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36,$AC36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC36" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="AC36" s="4">
+        <v>100</v>
+      </c>
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A37" s="5">
@@ -4011,64 +4269,64 @@
         <v>7</v>
       </c>
       <c r="E54" s="10">
-        <f>SUM(D14:D35)</f>
-        <v>35</v>
+        <f>SUM(D14:D51)</f>
+        <v>40</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H54" s="10">
-        <f>SUM(G14:G35)</f>
-        <v>-85</v>
+        <f>SUM(G14:G51)</f>
+        <v>-95</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K54" s="10">
-        <f>SUM(J14:J35)</f>
-        <v>80</v>
+        <f>SUM(J14:J51)</f>
+        <v>75</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N54" s="10">
-        <f>SUM(M14:M35)</f>
-        <v>35</v>
+        <f>SUM(M14:M51)</f>
+        <v>10</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q54" s="10">
-        <f>SUM(P14:P35)</f>
-        <v>-20</v>
+        <f>SUM(P14:P51)</f>
+        <v>0</v>
       </c>
       <c r="S54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T54" s="10">
-        <f>SUM(S14:S35)</f>
-        <v>55</v>
+        <f>SUM(S14:S51)</f>
+        <v>35</v>
       </c>
       <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W54" s="10">
-        <f>SUM(V14:V35)</f>
-        <v>7.5</v>
+        <f>SUM(V14:V51)</f>
+        <v>-7.5</v>
       </c>
       <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z54" s="10">
-        <f>SUM(Y14:Y35)</f>
+        <f>SUM(Y14:Y51)</f>
         <v>-225</v>
       </c>
       <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC54" s="10">
-        <f>SUM(AB14:AB35)</f>
-        <v>117.5</v>
+        <f>SUM(AB14:AB51)</f>
+        <v>167.5</v>
       </c>
       <c r="AD54" s="1">
         <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
@@ -4090,13 +4348,13 @@
     <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E54">
-    <cfRule type="cellIs" dxfId="26" priority="172" operator="lessThan">
+    <cfRule type="cellIs" dxfId="50" priority="196" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="173" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="197" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="174" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="198" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
24	1	RCB vs DC
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B67C5E-D9CE-C447-8552-B1CD54F1D4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE0342C-E271-B947-A1EA-C9C774EA9333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -465,8 +465,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -474,15 +474,25 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="51">
+  <dxfs count="27">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -490,6 +500,126 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -620,376 +750,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1340,24 +1100,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1366,22 +1126,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1390,22 +1150,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1414,22 +1174,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1438,22 +1198,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1462,22 +1222,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1486,22 +1246,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1510,22 +1270,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1540,10 +1300,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="22"/>
+      <c r="E12" s="19"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -3344,51 +3104,67 @@
       <c r="C37" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D37" s="3" t="str">
+      <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E37" s="4"/>
-      <c r="G37" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E37" s="4">
+        <v>90</v>
+      </c>
+      <c r="G37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H37" s="4"/>
-      <c r="J37" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H37" s="4">
+        <v>60</v>
+      </c>
+      <c r="J37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K37" s="4"/>
-      <c r="M37" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K37" s="4">
+        <v>30</v>
+      </c>
+      <c r="M37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N37" s="4"/>
-      <c r="P37" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N37" s="4">
+        <v>40</v>
+      </c>
+      <c r="P37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q37" s="4"/>
-      <c r="S37" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T37" s="4"/>
-      <c r="V37" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q37" s="4">
+        <v>100</v>
+      </c>
+      <c r="S37" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="T37" s="4">
+        <v>80</v>
+      </c>
+      <c r="V37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W37" s="4"/>
-      <c r="Y37" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W37" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z37" s="4"/>
-      <c r="AB37" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(AC37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37,$AC37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC37" s="4"/>
+        <v>-10</v>
+      </c>
+      <c r="Z37" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB37" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="AC37" s="4">
+        <v>80</v>
+      </c>
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
@@ -4270,63 +4046,63 @@
       </c>
       <c r="E54" s="10">
         <f>SUM(D14:D51)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H54" s="10">
         <f>SUM(G14:G51)</f>
-        <v>-95</v>
+        <v>-100</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K54" s="10">
         <f>SUM(J14:J51)</f>
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N54" s="10">
         <f>SUM(M14:M51)</f>
-        <v>10</v>
+        <v>-5</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q54" s="10">
         <f>SUM(P14:P51)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="S54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T54" s="10">
         <f>SUM(S14:S51)</f>
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W54" s="10">
         <f>SUM(V14:V51)</f>
-        <v>-7.5</v>
+        <v>-32.5</v>
       </c>
       <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z54" s="10">
         <f>SUM(Y14:Y51)</f>
-        <v>-225</v>
+        <v>-235</v>
       </c>
       <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC54" s="10">
         <f>SUM(AB14:AB51)</f>
-        <v>167.5</v>
+        <v>170</v>
       </c>
       <c r="AD54" s="1">
         <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
@@ -4336,66 +4112,66 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E54">
-    <cfRule type="cellIs" dxfId="50" priority="196" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="198" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="197" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="197" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="198" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="196" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H54">
-    <cfRule type="cellIs" dxfId="23" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K54">
-    <cfRule type="cellIs" dxfId="20" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N54">
-    <cfRule type="cellIs" dxfId="17" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q54">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
@@ -4403,46 +4179,46 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T54">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W54">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z54">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC54">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
ontest 25: CSK vs KKR Contest 26: LSG vs GT Contest 27: SRH vs PBKS Contest 28: RR vs RCB Contest 29: DC vs MI
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE0342C-E271-B947-A1EA-C9C774EA9333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C17507-864F-444B-B0A2-0738BF0D4138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -465,8 +465,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -474,8 +474,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1100,24 +1100,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1126,22 +1126,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1150,22 +1150,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1174,22 +1174,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1198,22 +1198,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1222,22 +1222,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1246,22 +1246,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1270,22 +1270,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1300,10 +1300,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="19"/>
+      <c r="E12" s="22"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -3176,51 +3176,66 @@
       <c r="C38" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D38" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E38" s="4"/>
-      <c r="G38" s="3" t="str">
+      <c r="D38" s="3">
+        <v>-20</v>
+      </c>
+      <c r="E38" s="4">
+        <v>40</v>
+      </c>
+      <c r="G38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H38" s="4"/>
-      <c r="J38" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H38" s="4">
+        <v>100</v>
+      </c>
+      <c r="J38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K38" s="4"/>
-      <c r="M38" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K38" s="4">
+        <v>90</v>
+      </c>
+      <c r="M38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N38" s="4"/>
-      <c r="P38" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N38" s="4">
+        <v>60</v>
+      </c>
+      <c r="P38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q38" s="4"/>
-      <c r="S38" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q38" s="4">
+        <v>80</v>
+      </c>
+      <c r="S38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T38" s="4"/>
-      <c r="V38" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W38" s="4"/>
-      <c r="Y38" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z38" s="4"/>
-      <c r="AB38" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="T38" s="4">
+        <v>70</v>
+      </c>
+      <c r="V38" s="3">
+        <v>-20</v>
+      </c>
+      <c r="W38" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y38" s="3">
+        <v>-20</v>
+      </c>
+      <c r="Z38" s="4">
+        <v>40</v>
+      </c>
+      <c r="AB38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38,$AC38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC38" s="4"/>
+        <v>-10</v>
+      </c>
+      <c r="AC38" s="4">
+        <v>50</v>
+      </c>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A39" s="5">
@@ -3232,51 +3247,67 @@
       <c r="C39" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D39" s="3" t="str">
+      <c r="D39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E39" s="4"/>
-      <c r="G39" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E39" s="4">
+        <v>100</v>
+      </c>
+      <c r="G39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H39" s="4"/>
-      <c r="J39" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H39" s="4">
+        <v>60</v>
+      </c>
+      <c r="J39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K39" s="4"/>
-      <c r="M39" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N39" s="4"/>
-      <c r="P39" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K39" s="4">
+        <v>90</v>
+      </c>
+      <c r="M39" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="N39" s="4">
+        <v>30</v>
+      </c>
+      <c r="P39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q39" s="4"/>
-      <c r="S39" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q39" s="4">
+        <v>80</v>
+      </c>
+      <c r="S39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T39" s="4"/>
-      <c r="V39" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T39" s="4">
+        <v>50</v>
+      </c>
+      <c r="V39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W39" s="4"/>
-      <c r="Y39" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z39" s="4"/>
-      <c r="AB39" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W39" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y39" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="Z39" s="4">
+        <v>30</v>
+      </c>
+      <c r="AB39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39,$AC39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC39" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC39" s="4">
+        <v>70</v>
+      </c>
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
@@ -3288,51 +3319,67 @@
       <c r="C40" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D40" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E40" s="4"/>
-      <c r="G40" s="3" t="str">
+      <c r="D40" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E40" s="4">
+        <v>30</v>
+      </c>
+      <c r="G40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H40" s="4"/>
-      <c r="J40" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K40" s="4"/>
-      <c r="M40" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4">
+        <v>70</v>
+      </c>
+      <c r="J40" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="K40" s="4">
+        <v>30</v>
+      </c>
+      <c r="M40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N40" s="4"/>
-      <c r="P40" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N40" s="4">
+        <v>40</v>
+      </c>
+      <c r="P40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q40" s="4"/>
-      <c r="S40" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>100</v>
+      </c>
+      <c r="S40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T40" s="4"/>
-      <c r="V40" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T40" s="4">
+        <v>80</v>
+      </c>
+      <c r="V40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W40" s="4"/>
-      <c r="Y40" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W40" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z40" s="4"/>
-      <c r="AB40" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Z40" s="4">
+        <v>60</v>
+      </c>
+      <c r="AB40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40,$AC40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC40" s="4"/>
+        <v>-10</v>
+      </c>
+      <c r="AC40" s="4">
+        <v>50</v>
+      </c>
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A41" s="5">
@@ -3344,51 +3391,67 @@
       <c r="C41" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E41" s="4"/>
-      <c r="G41" s="3" t="str">
+      <c r="D41" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E41" s="4">
+        <v>30</v>
+      </c>
+      <c r="G41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H41" s="4"/>
-      <c r="J41" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H41" s="4">
+        <v>80</v>
+      </c>
+      <c r="J41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K41" s="4"/>
-      <c r="M41" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N41" s="4"/>
-      <c r="P41" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K41" s="4">
+        <v>60</v>
+      </c>
+      <c r="M41" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="N41" s="4">
+        <v>30</v>
+      </c>
+      <c r="P41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q41" s="4"/>
-      <c r="S41" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="4">
+        <v>70</v>
+      </c>
+      <c r="S41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T41" s="4"/>
-      <c r="V41" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T41" s="4">
+        <v>90</v>
+      </c>
+      <c r="V41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W41" s="4"/>
-      <c r="Y41" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W41" s="4">
+        <v>100</v>
+      </c>
+      <c r="Y41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z41" s="4"/>
-      <c r="AB41" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Z41" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41,$AC41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC41" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="AC41" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
@@ -3400,51 +3463,69 @@
       <c r="C42" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D42" s="3" t="str">
+      <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E42" s="4"/>
-      <c r="G42" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="E42" s="4">
+        <v>30</v>
+      </c>
+      <c r="G42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H42" s="4"/>
-      <c r="J42" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H42" s="4">
+        <v>40</v>
+      </c>
+      <c r="J42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K42" s="4"/>
-      <c r="M42" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K42" s="4">
+        <v>50</v>
+      </c>
+      <c r="M42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N42" s="4"/>
-      <c r="P42" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N42" s="4">
+        <v>0</v>
+      </c>
+      <c r="P42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q42" s="4"/>
-      <c r="S42" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="4">
+        <v>70</v>
+      </c>
+      <c r="S42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T42" s="4"/>
-      <c r="V42" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T42" s="4">
+        <v>100</v>
+      </c>
+      <c r="V42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W42" s="4"/>
-      <c r="Y42" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W42" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z42" s="4"/>
-      <c r="AB42" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z42" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42,$AC42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC42" s="4"/>
+        <v>-5</v>
+      </c>
+      <c r="AC42" s="4">
+        <v>60</v>
+      </c>
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A43" s="5">
@@ -4046,63 +4127,63 @@
       </c>
       <c r="E54" s="10">
         <f>SUM(D14:D51)</f>
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H54" s="10">
         <f>SUM(G14:G51)</f>
-        <v>-100</v>
+        <v>-65</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K54" s="10">
         <f>SUM(J14:J51)</f>
-        <v>55</v>
+        <v>57.5</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N54" s="10">
         <f>SUM(M14:M51)</f>
-        <v>-5</v>
+        <v>-95</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q54" s="10">
         <f>SUM(P14:P51)</f>
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="S54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T54" s="10">
         <f>SUM(S14:S51)</f>
-        <v>37.5</v>
+        <v>102.5</v>
       </c>
       <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W54" s="10">
         <f>SUM(V14:V51)</f>
-        <v>-32.5</v>
+        <v>22.5</v>
       </c>
       <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z54" s="10">
         <f>SUM(Y14:Y51)</f>
-        <v>-235</v>
+        <v>-287.5</v>
       </c>
       <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC54" s="10">
         <f>SUM(AB14:AB51)</f>
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="AD54" s="1">
         <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
@@ -4112,16 +4193,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
   <conditionalFormatting sqref="E54">
     <cfRule type="cellIs" dxfId="26" priority="198" operator="greaterThan">

</xml_diff>

<commit_message>
31 pbks vs kkr
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3591C266-4403-014E-B3DC-2E3AFE06A80B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053B3DFB-574D-8F4E-84D8-BB80062AF75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -465,8 +465,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -474,8 +474,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1100,24 +1100,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1126,22 +1126,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1150,22 +1150,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1174,22 +1174,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1198,22 +1198,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1222,22 +1222,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1246,22 +1246,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1270,22 +1270,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1300,10 +1300,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="22"/>
+      <c r="E12" s="19"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -3611,51 +3611,69 @@
       <c r="C44" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="3" t="str">
+      <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E44" s="4"/>
-      <c r="G44" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E44" s="4">
+        <v>100</v>
+      </c>
+      <c r="G44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H44" s="4"/>
-      <c r="J44" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H44" s="4">
+        <v>90</v>
+      </c>
+      <c r="J44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K44" s="4"/>
-      <c r="M44" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K44" s="4">
+        <v>60</v>
+      </c>
+      <c r="M44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N44" s="4"/>
-      <c r="P44" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N44" s="4">
+        <v>0</v>
+      </c>
+      <c r="P44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q44" s="4"/>
-      <c r="S44" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="4">
+        <v>70</v>
+      </c>
+      <c r="S44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T44" s="4"/>
-      <c r="V44" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T44" s="4">
+        <v>50</v>
+      </c>
+      <c r="V44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W44" s="4"/>
-      <c r="Y44" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W44" s="4">
+        <v>30</v>
+      </c>
+      <c r="Y44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z44" s="4"/>
-      <c r="AB44" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z44" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44,$AC44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC44" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="AC44" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="45" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A45" s="5">
@@ -4145,28 +4163,28 @@
       </c>
       <c r="E54" s="10">
         <f>SUM(D14:D51)</f>
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H54" s="10">
         <f>SUM(G14:G51)</f>
-        <v>-60</v>
+        <v>-40</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K54" s="10">
         <f>SUM(J14:J51)</f>
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N54" s="10">
         <f>SUM(M14:M51)</f>
-        <v>-105</v>
+        <v>-130</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>7</v>
@@ -4180,28 +4198,28 @@
       </c>
       <c r="T54" s="10">
         <f>SUM(S14:S51)</f>
-        <v>122.5</v>
+        <v>112.5</v>
       </c>
       <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W54" s="10">
         <f>SUM(V14:V51)</f>
-        <v>2.5</v>
+        <v>-17.5</v>
       </c>
       <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z54" s="10">
         <f>SUM(Y14:Y51)</f>
-        <v>-292.5</v>
+        <v>-287.5</v>
       </c>
       <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC54" s="10">
         <f>SUM(AB14:AB51)</f>
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="AD54" s="1">
         <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
@@ -4211,16 +4229,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E54">
     <cfRule type="cellIs" dxfId="26" priority="198" operator="greaterThan">

</xml_diff>

<commit_message>
Contest 32: DC vs RR
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053B3DFB-574D-8F4E-84D8-BB80062AF75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DBC0E6-5BC5-194C-8D55-DE61BFC325C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -465,8 +465,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -474,8 +474,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1100,24 +1100,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1126,22 +1126,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1150,22 +1150,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1174,22 +1174,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1198,22 +1198,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1222,22 +1222,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1246,22 +1246,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1270,22 +1270,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1300,10 +1300,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="19"/>
+      <c r="E12" s="22"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -3685,51 +3685,67 @@
       <c r="C45" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E45" s="4"/>
-      <c r="G45" s="3" t="str">
+      <c r="D45" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E45" s="4">
+        <v>30</v>
+      </c>
+      <c r="G45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H45" s="4"/>
-      <c r="J45" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="H45" s="4">
+        <v>70</v>
+      </c>
+      <c r="J45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K45" s="4"/>
-      <c r="M45" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K45" s="4">
+        <v>40</v>
+      </c>
+      <c r="M45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N45" s="4"/>
-      <c r="P45" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N45" s="4">
+        <v>100</v>
+      </c>
+      <c r="P45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q45" s="4"/>
-      <c r="S45" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q45" s="4">
+        <v>50</v>
+      </c>
+      <c r="S45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T45" s="4"/>
-      <c r="V45" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W45" s="4"/>
-      <c r="Y45" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T45" s="4">
+        <v>60</v>
+      </c>
+      <c r="V45" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="W45" s="4">
+        <v>30</v>
+      </c>
+      <c r="Y45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z45" s="4"/>
-      <c r="AB45" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Z45" s="4">
+        <v>90</v>
+      </c>
+      <c r="AB45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45,$AC45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC45" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="AC45" s="4">
+        <v>80</v>
+      </c>
     </row>
     <row r="46" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
@@ -4163,7 +4179,7 @@
       </c>
       <c r="E54" s="10">
         <f>SUM(D14:D51)</f>
-        <v>125</v>
+        <v>102.5</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>7</v>
@@ -4177,49 +4193,49 @@
       </c>
       <c r="K54" s="10">
         <f>SUM(J14:J51)</f>
-        <v>27.5</v>
+        <v>12.5</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N54" s="10">
         <f>SUM(M14:M51)</f>
-        <v>-130</v>
+        <v>-80</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q54" s="10">
         <f>SUM(P14:P51)</f>
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="S54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T54" s="10">
         <f>SUM(S14:S51)</f>
-        <v>112.5</v>
+        <v>107.5</v>
       </c>
       <c r="V54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W54" s="10">
         <f>SUM(V14:V51)</f>
-        <v>-17.5</v>
+        <v>-40</v>
       </c>
       <c r="Y54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z54" s="10">
         <f>SUM(Y14:Y51)</f>
-        <v>-287.5</v>
+        <v>-267.5</v>
       </c>
       <c r="AB54" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC54" s="10">
         <f>SUM(AB14:AB51)</f>
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="AD54" s="1">
         <f>SUM(E54,H54,K54,N54,Q54,T54,W54,Z54,AC54)</f>
@@ -4229,16 +4245,16 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
   <conditionalFormatting sqref="E54">
     <cfRule type="cellIs" dxfId="26" priority="198" operator="greaterThan">

</xml_diff>

<commit_message>
new match entries after 38
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795740A8-C7BB-FA44-A0FE-1EFD847E8A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C6E99F-26D3-6C4F-A943-BE418903359E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="91">
   <si>
     <t>Points</t>
   </si>
@@ -267,6 +267,54 @@
   </si>
   <si>
     <t>MI vs CSK</t>
+  </si>
+  <si>
+    <t>KKR vs GT</t>
+  </si>
+  <si>
+    <t>LSG vs DC</t>
+  </si>
+  <si>
+    <t>SRH vs MI</t>
+  </si>
+  <si>
+    <t>RCB vs RR</t>
+  </si>
+  <si>
+    <t>CSK vs SRH</t>
+  </si>
+  <si>
+    <t>KKR vs PBKS</t>
+  </si>
+  <si>
+    <t>MI vs LSH</t>
+  </si>
+  <si>
+    <t>DC vs RCB</t>
+  </si>
+  <si>
+    <t>RR vs GT</t>
+  </si>
+  <si>
+    <t>DC vs KKR</t>
+  </si>
+  <si>
+    <t>CSK vs PBKS</t>
+  </si>
+  <si>
+    <t>RR vs MI</t>
+  </si>
+  <si>
+    <t>GT vs SRH</t>
+  </si>
+  <si>
+    <t>RCB vs CSK</t>
+  </si>
+  <si>
+    <t>KKR vs RR</t>
+  </si>
+  <si>
+    <t>PBKS vs LSG</t>
   </si>
 </sst>
 </file>
@@ -4193,7 +4241,9 @@
       <c r="B52" s="4">
         <v>1</v>
       </c>
-      <c r="C52" s="18"/>
+      <c r="C52" s="18" t="s">
+        <v>75</v>
+      </c>
       <c r="D52" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4247,7 +4297,9 @@
       <c r="B53" s="4">
         <v>1</v>
       </c>
-      <c r="C53" s="18"/>
+      <c r="C53" s="18" t="s">
+        <v>76</v>
+      </c>
       <c r="D53" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53,$AC53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53,$AC53), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4301,7 +4353,9 @@
       <c r="B54" s="4">
         <v>1</v>
       </c>
-      <c r="C54" s="18"/>
+      <c r="C54" s="18" t="s">
+        <v>77</v>
+      </c>
       <c r="D54" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54,$AC54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54,$AC54), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4355,7 +4409,9 @@
       <c r="B55" s="4">
         <v>1</v>
       </c>
-      <c r="C55" s="18"/>
+      <c r="C55" s="18" t="s">
+        <v>78</v>
+      </c>
       <c r="D55" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55,$AC55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55,$AC55), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4409,7 +4465,9 @@
       <c r="B56" s="4">
         <v>1</v>
       </c>
-      <c r="C56" s="18"/>
+      <c r="C56" s="18" t="s">
+        <v>79</v>
+      </c>
       <c r="D56" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56,$AC56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56,$AC56), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4463,7 +4521,9 @@
       <c r="B57" s="4">
         <v>1</v>
       </c>
-      <c r="C57" s="18"/>
+      <c r="C57" s="18" t="s">
+        <v>80</v>
+      </c>
       <c r="D57" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57,$AC57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57,$AC57), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4517,7 +4577,9 @@
       <c r="B58" s="4">
         <v>1</v>
       </c>
-      <c r="C58" s="18"/>
+      <c r="C58" s="18" t="s">
+        <v>81</v>
+      </c>
       <c r="D58" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58,$AC58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58,$AC58), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4571,7 +4633,9 @@
       <c r="B59" s="4">
         <v>1</v>
       </c>
-      <c r="C59" s="18"/>
+      <c r="C59" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="D59" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59,$AC59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59,$AC59), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4625,7 +4689,9 @@
       <c r="B60" s="4">
         <v>1</v>
       </c>
-      <c r="C60" s="18"/>
+      <c r="C60" s="18" t="s">
+        <v>83</v>
+      </c>
       <c r="D60" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60,$AC60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60,$AC60), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4679,7 +4745,9 @@
       <c r="B61" s="4">
         <v>1</v>
       </c>
-      <c r="C61" s="18"/>
+      <c r="C61" s="18" t="s">
+        <v>84</v>
+      </c>
       <c r="D61" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61,$AC61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61,$AC61), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4733,7 +4801,9 @@
       <c r="B62" s="4">
         <v>1</v>
       </c>
-      <c r="C62" s="18"/>
+      <c r="C62" s="18" t="s">
+        <v>85</v>
+      </c>
       <c r="D62" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62,$AC62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62,$AC62), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4787,7 +4857,9 @@
       <c r="B63" s="4">
         <v>1</v>
       </c>
-      <c r="C63" s="18"/>
+      <c r="C63" s="18" t="s">
+        <v>86</v>
+      </c>
       <c r="D63" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63,$AC63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63,$AC63), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4841,7 +4913,9 @@
       <c r="B64" s="4">
         <v>1</v>
       </c>
-      <c r="C64" s="18"/>
+      <c r="C64" s="18" t="s">
+        <v>87</v>
+      </c>
       <c r="D64" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64,$AC64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64,$AC64), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4895,7 +4969,9 @@
       <c r="B65" s="4">
         <v>1</v>
       </c>
-      <c r="C65" s="18"/>
+      <c r="C65" s="18" t="s">
+        <v>88</v>
+      </c>
       <c r="D65" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65,$AC65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65,$AC65), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4949,7 +5025,9 @@
       <c r="B66" s="4">
         <v>1</v>
       </c>
-      <c r="C66" s="18"/>
+      <c r="C66" s="18" t="s">
+        <v>89</v>
+      </c>
       <c r="D66" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66,$AC66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66,$AC66), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -5003,7 +5081,9 @@
       <c r="B67" s="4">
         <v>1</v>
       </c>
-      <c r="C67" s="18"/>
+      <c r="C67" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="D67" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67,$AC67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67,$AC67), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>

</xml_diff>

<commit_message>
39 kkr vs gt
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C6E99F-26D3-6C4F-A943-BE418903359E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E12AB32-927F-1146-8ABC-486760E8FC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -513,8 +513,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -522,15 +522,25 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="51">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -798,6 +808,236 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1148,24 +1388,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1174,22 +1414,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1198,22 +1438,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1222,22 +1462,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1246,22 +1486,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1270,22 +1510,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1294,22 +1534,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
-      <c r="S8" s="19"/>
-      <c r="T8" s="19"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="19"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1318,22 +1558,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1348,10 +1588,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="22"/>
+      <c r="E12" s="19"/>
       <c r="G12" s="20" t="s">
         <v>13</v>
       </c>
@@ -4244,51 +4484,69 @@
       <c r="C52" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D52" s="3" t="str">
+      <c r="D52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E52" s="4"/>
-      <c r="G52" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E52" s="4">
+        <v>0</v>
+      </c>
+      <c r="G52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H52" s="4"/>
-      <c r="J52" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H52" s="4">
+        <v>40</v>
+      </c>
+      <c r="J52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K52" s="4"/>
-      <c r="M52" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K52" s="4">
+        <v>80</v>
+      </c>
+      <c r="M52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N52" s="4"/>
-      <c r="P52" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N52" s="4">
+        <v>30</v>
+      </c>
+      <c r="P52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q52" s="4"/>
-      <c r="S52" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q52" s="4">
+        <v>90</v>
+      </c>
+      <c r="S52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T52" s="4"/>
-      <c r="V52" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T52" s="4">
+        <v>50</v>
+      </c>
+      <c r="V52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W52" s="4"/>
-      <c r="Y52" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W52" s="4">
+        <v>100</v>
+      </c>
+      <c r="Y52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z52" s="4"/>
-      <c r="AB52" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="4">
+        <v>70</v>
+      </c>
+      <c r="AB52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52,$AC52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC52" s="4"/>
+        <v>-5</v>
+      </c>
+      <c r="AC52" s="4">
+        <v>60</v>
+      </c>
     </row>
     <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53" s="5">
@@ -5225,64 +5483,64 @@
         <v>7</v>
       </c>
       <c r="E70" s="10">
-        <f>SUM(D14:D51)</f>
-        <v>50</v>
+        <f>SUM(D14:D67)</f>
+        <v>25</v>
       </c>
       <c r="G70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H70" s="10">
-        <f>SUM(G14:G51)</f>
-        <v>5</v>
+        <f>SUM(G14:G67)</f>
+        <v>-10</v>
       </c>
       <c r="J70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K70" s="10">
-        <f>SUM(J14:J51)</f>
-        <v>-42.5</v>
+        <f>SUM(J14:J67)</f>
+        <v>-37.5</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N70" s="10">
-        <f>SUM(M14:M51)</f>
-        <v>7.5</v>
+        <f>SUM(M14:M67)</f>
+        <v>-12.5</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q70" s="10">
-        <f>SUM(P14:P51)</f>
-        <v>175</v>
+        <f>SUM(P14:P67)</f>
+        <v>195</v>
       </c>
       <c r="S70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T70" s="10">
-        <f>SUM(S14:S51)</f>
-        <v>42.5</v>
+        <f>SUM(S14:S67)</f>
+        <v>32.5</v>
       </c>
       <c r="V70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W70" s="10">
-        <f>SUM(V14:V51)</f>
-        <v>-85</v>
+        <f>SUM(V14:V67)</f>
+        <v>-35</v>
       </c>
       <c r="Y70" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z70" s="10">
-        <f>SUM(Y14:Y51)</f>
+        <f>SUM(Y14:Y67)</f>
         <v>-262.5</v>
       </c>
       <c r="AB70" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC70" s="10">
-        <f>SUM(AB14:AB51)</f>
-        <v>110</v>
+        <f>SUM(AB14:AB67)</f>
+        <v>105</v>
       </c>
       <c r="AD70" s="1">
         <f>SUM(E70,H70,K70,N70,Q70,T70,W70,Z70,AC70)</f>
@@ -5292,113 +5550,113 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="10">
+    <mergeCell ref="I2:X9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="I2:X9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="Y12:Z12"/>
   </mergeCells>
   <conditionalFormatting sqref="E70">
-    <cfRule type="cellIs" dxfId="26" priority="196" operator="lessThan">
+    <cfRule type="cellIs" dxfId="50" priority="222" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="197" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="221" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="198" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="220" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H70">
-    <cfRule type="cellIs" dxfId="23" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K70">
-    <cfRule type="cellIs" dxfId="20" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N70">
-    <cfRule type="cellIs" dxfId="17" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q70">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T70">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W70">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z70">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC70">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
qualifier 1: pbks vs rcb
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED6932A-04A8-4B4A-B792-5977F28892A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBDB813-A83D-1946-8501-AF3C5F6CC1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="124">
   <si>
     <t>Points</t>
   </si>
@@ -366,13 +366,61 @@
   </si>
   <si>
     <t>LSG vs RCB</t>
+  </si>
+  <si>
+    <t>Qualifier 1</t>
+  </si>
+  <si>
+    <t>Eliminator</t>
+  </si>
+  <si>
+    <t>Qualifier 2</t>
+  </si>
+  <si>
+    <t>Finals</t>
+  </si>
+  <si>
+    <t>Winner Prediction - Coins</t>
+  </si>
+  <si>
+    <t>Scorecard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finals </t>
+  </si>
+  <si>
+    <t>Format 1</t>
+  </si>
+  <si>
+    <t>Format 2</t>
+  </si>
+  <si>
+    <t>Total coins</t>
+  </si>
+  <si>
+    <t>Outgoing</t>
+  </si>
+  <si>
+    <t>Coins</t>
+  </si>
+  <si>
+    <t>Incoming</t>
+  </si>
+  <si>
+    <t>Format 3</t>
+  </si>
+  <si>
+    <t>Format 4</t>
+  </si>
+  <si>
+    <t>Format 5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -419,8 +467,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -457,8 +526,19 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -531,12 +611,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -567,8 +659,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -576,25 +668,53 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="33">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -602,126 +722,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -852,6 +852,196 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1170,18 +1360,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE9CB7-B9A7-B347-86F0-C3EB9B5BFBBD}">
-  <dimension ref="A1:AD86"/>
+  <dimension ref="A1:AD108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3.5" customWidth="1"/>
+    <col min="4" max="4" width="8.1640625" customWidth="1"/>
+    <col min="5" max="5" width="9.5" customWidth="1"/>
+    <col min="6" max="7" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="8.6640625" customWidth="1"/>
     <col min="12" max="12" width="3" customWidth="1"/>
     <col min="15" max="15" width="2.83203125" customWidth="1"/>
-    <col min="18" max="18" width="2.83203125" customWidth="1"/>
-    <col min="21" max="21" width="2.83203125" customWidth="1"/>
+    <col min="18" max="18" width="9.1640625" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" customWidth="1"/>
     <col min="24" max="24" width="2.1640625" customWidth="1"/>
     <col min="27" max="27" width="4.1640625" customWidth="1"/>
   </cols>
@@ -1202,24 +1393,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+      <c r="S2" s="20"/>
+      <c r="T2" s="20"/>
+      <c r="U2" s="20"/>
+      <c r="V2" s="20"/>
+      <c r="W2" s="20"/>
+      <c r="X2" s="20"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1228,22 +1419,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="23"/>
-      <c r="Q3" s="23"/>
-      <c r="R3" s="23"/>
-      <c r="S3" s="23"/>
-      <c r="T3" s="23"/>
-      <c r="U3" s="23"/>
-      <c r="V3" s="23"/>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="20"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1252,22 +1443,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="23"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20"/>
+      <c r="X4" s="20"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1276,22 +1467,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
-      <c r="T5" s="23"/>
-      <c r="U5" s="23"/>
-      <c r="V5" s="23"/>
-      <c r="W5" s="23"/>
-      <c r="X5" s="23"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20"/>
+      <c r="X5" s="20"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1300,22 +1491,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="23"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="23"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="23"/>
-      <c r="X6" s="23"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
+      <c r="U6" s="20"/>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20"/>
+      <c r="X6" s="20"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1324,22 +1515,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="23"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="23"/>
-      <c r="T7" s="23"/>
-      <c r="U7" s="23"/>
-      <c r="V7" s="23"/>
-      <c r="W7" s="23"/>
-      <c r="X7" s="23"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
+      <c r="X7" s="20"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1348,22 +1539,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="23"/>
-      <c r="Q8" s="23"/>
-      <c r="R8" s="23"/>
-      <c r="S8" s="23"/>
-      <c r="T8" s="23"/>
-      <c r="U8" s="23"/>
-      <c r="V8" s="23"/>
-      <c r="W8" s="23"/>
-      <c r="X8" s="23"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20"/>
+      <c r="X8" s="20"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1372,22 +1563,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="23"/>
-      <c r="S9" s="23"/>
-      <c r="T9" s="23"/>
-      <c r="U9" s="23"/>
-      <c r="V9" s="23"/>
-      <c r="W9" s="23"/>
-      <c r="X9" s="23"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
+      <c r="T9" s="20"/>
+      <c r="U9" s="20"/>
+      <c r="V9" s="20"/>
+      <c r="W9" s="20"/>
+      <c r="X9" s="20"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1402,10 +1593,10 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="20"/>
+      <c r="E12" s="23"/>
       <c r="G12" s="21" t="s">
         <v>13</v>
       </c>
@@ -6528,321 +6719,1148 @@
       <c r="C83" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D83" s="3" t="str">
+      <c r="D83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-5</v>
+      </c>
+      <c r="E83" s="4">
+        <v>60</v>
+      </c>
+      <c r="G83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>5</v>
+      </c>
+      <c r="H83" s="4">
+        <v>80</v>
+      </c>
+      <c r="J83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>20</v>
+      </c>
+      <c r="K83" s="4">
+        <v>90</v>
+      </c>
+      <c r="M83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>0</v>
+      </c>
+      <c r="N83" s="4">
+        <v>70</v>
+      </c>
+      <c r="P83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-25</v>
+      </c>
+      <c r="Q83" s="4">
+        <v>0</v>
+      </c>
+      <c r="S83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-15</v>
+      </c>
+      <c r="T83" s="4">
+        <v>40</v>
+      </c>
+      <c r="V83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-10</v>
+      </c>
+      <c r="W83" s="4">
+        <v>50</v>
+      </c>
+      <c r="Y83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>50</v>
+      </c>
+      <c r="Z83" s="4">
+        <v>100</v>
+      </c>
+      <c r="AB83" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-20</v>
+      </c>
+      <c r="AC83" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="84" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A84" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B84" s="4">
+        <v>1</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-20</v>
+      </c>
+      <c r="E84" s="4">
+        <v>30</v>
+      </c>
+      <c r="G84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>50</v>
+      </c>
+      <c r="H84" s="4">
+        <v>100</v>
+      </c>
+      <c r="J84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-25</v>
+      </c>
+      <c r="K84" s="4">
+        <v>0</v>
+      </c>
+      <c r="M84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>20</v>
+      </c>
+      <c r="N84" s="4">
+        <v>90</v>
+      </c>
+      <c r="P84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-15</v>
+      </c>
+      <c r="Q84" s="4">
+        <v>40</v>
+      </c>
+      <c r="S84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>0</v>
+      </c>
+      <c r="T84" s="4">
+        <v>70</v>
+      </c>
+      <c r="V84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>5</v>
+      </c>
+      <c r="W84" s="4">
+        <v>80</v>
+      </c>
+      <c r="Y84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-10</v>
+      </c>
+      <c r="Z84" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84,$AC84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-5</v>
+      </c>
+      <c r="AC84" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="85" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A85" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B85" s="4">
+        <v>1</v>
+      </c>
+      <c r="C85" s="18"/>
+      <c r="D85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="E83" s="4"/>
-      <c r="G83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="E85" s="4"/>
+      <c r="G85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="H83" s="4"/>
-      <c r="J83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="H85" s="4"/>
+      <c r="J85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="K83" s="4"/>
-      <c r="M83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="K85" s="4"/>
+      <c r="M85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="N83" s="4"/>
-      <c r="P83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="N85" s="4"/>
+      <c r="P85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="Q83" s="4"/>
-      <c r="S83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="Q85" s="4"/>
+      <c r="S85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="T83" s="4"/>
-      <c r="V83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="T85" s="4"/>
+      <c r="V85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="W83" s="4"/>
-      <c r="Y83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="W85" s="4"/>
+      <c r="Y85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="Z83" s="4"/>
-      <c r="AB83" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(AC83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83,$AC83), 0),  $A$2:$B$10, 2, FALSE))</f>
+      <c r="Z85" s="4"/>
+      <c r="AB85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
       </c>
-      <c r="AC83" s="4"/>
-    </row>
-    <row r="84" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A84" s="5"/>
-      <c r="B84" s="1" t="s">
+      <c r="AC85" s="4"/>
+    </row>
+    <row r="86" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A86" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" s="4">
+        <v>1</v>
+      </c>
+      <c r="C86" s="18"/>
+      <c r="D86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E86" s="4"/>
+      <c r="G86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H86" s="4"/>
+      <c r="J86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K86" s="4"/>
+      <c r="M86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N86" s="4"/>
+      <c r="P86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q86" s="4"/>
+      <c r="S86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T86" s="4"/>
+      <c r="V86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W86" s="4"/>
+      <c r="Y86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z86" s="4"/>
+      <c r="AB86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC86" s="4"/>
+    </row>
+    <row r="87" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A87" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B87" s="4">
+        <v>1</v>
+      </c>
+      <c r="C87" s="18"/>
+      <c r="D87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E87" s="4"/>
+      <c r="G87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H87" s="4"/>
+      <c r="J87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K87" s="4"/>
+      <c r="M87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N87" s="4"/>
+      <c r="P87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q87" s="4"/>
+      <c r="S87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T87" s="4"/>
+      <c r="V87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W87" s="4"/>
+      <c r="Y87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z87" s="4"/>
+      <c r="AB87" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(AC87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="AC87" s="4"/>
+    </row>
+    <row r="88" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A88" s="5"/>
+      <c r="B88" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C84" s="8"/>
-      <c r="D84" s="1"/>
-      <c r="E84" s="7" t="s">
+      <c r="C88" s="8"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G84" s="1"/>
-      <c r="H84" s="7" t="s">
+      <c r="G88" s="1"/>
+      <c r="H88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="J84" s="1"/>
-      <c r="K84" s="7" t="s">
+      <c r="J88" s="1"/>
+      <c r="K88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="M84" s="1"/>
-      <c r="N84" s="7" t="s">
+      <c r="M88" s="1"/>
+      <c r="N88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="P84" s="1"/>
-      <c r="Q84" s="7" t="s">
+      <c r="P88" s="1"/>
+      <c r="Q88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="S84" s="1"/>
-      <c r="T84" s="7" t="s">
+      <c r="S88" s="1"/>
+      <c r="T88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="V84" s="1"/>
-      <c r="W84" s="7" t="s">
+      <c r="V88" s="1"/>
+      <c r="W88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="Y84" s="1"/>
-      <c r="Z84" s="7" t="s">
+      <c r="Y88" s="1"/>
+      <c r="Z88" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AB84" s="1"/>
-      <c r="AC84" s="7" t="s">
+      <c r="AB88" s="1"/>
+      <c r="AC88" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="D85" s="1"/>
-      <c r="E85" s="9" t="str">
+    <row r="89" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="D89" s="1"/>
+      <c r="E89" s="9" t="str">
         <f>D13</f>
         <v>Jaya</v>
       </c>
-      <c r="G85" s="1"/>
-      <c r="H85" s="9" t="str">
+      <c r="G89" s="1"/>
+      <c r="H89" s="9" t="str">
         <f>G13</f>
         <v>Justin</v>
       </c>
-      <c r="J85" s="1"/>
-      <c r="K85" s="9" t="str">
+      <c r="J89" s="1"/>
+      <c r="K89" s="9" t="str">
         <f>J13</f>
         <v>Ram</v>
       </c>
-      <c r="M85" s="1"/>
-      <c r="N85" s="9" t="str">
+      <c r="M89" s="1"/>
+      <c r="N89" s="9" t="str">
         <f>M13</f>
         <v>Sibi</v>
       </c>
-      <c r="P85" s="1"/>
-      <c r="Q85" s="9" t="str">
+      <c r="P89" s="1"/>
+      <c r="Q89" s="9" t="str">
         <f>P13</f>
         <v>Sundar</v>
       </c>
-      <c r="S85" s="1"/>
-      <c r="T85" s="9" t="str">
+      <c r="S89" s="1"/>
+      <c r="T89" s="9" t="str">
         <f>S13</f>
         <v>Sampath</v>
       </c>
-      <c r="V85" s="1"/>
-      <c r="W85" s="9" t="str">
+      <c r="V89" s="1"/>
+      <c r="W89" s="9" t="str">
         <f>V13</f>
         <v>Jayanth</v>
       </c>
-      <c r="Y85" s="1"/>
-      <c r="Z85" s="9" t="str">
+      <c r="Y89" s="1"/>
+      <c r="Z89" s="9" t="str">
         <f>Y13</f>
         <v>Vicky</v>
       </c>
-      <c r="AB85" s="1"/>
-      <c r="AC85" s="9" t="str">
+      <c r="AB89" s="1"/>
+      <c r="AC89" s="9" t="str">
         <f>AB13</f>
         <v>Anantha</v>
       </c>
     </row>
-    <row r="86" spans="1:30" ht="21" x14ac:dyDescent="0.25">
-      <c r="D86" s="6" t="s">
+    <row r="90" spans="1:30" ht="21" x14ac:dyDescent="0.25">
+      <c r="D90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E86" s="10">
-        <f>SUM(D14:D83)</f>
-        <v>-210</v>
-      </c>
-      <c r="G86" s="6" t="s">
+      <c r="E90" s="10">
+        <f>SUM(D14:D87)</f>
+        <v>-235</v>
+      </c>
+      <c r="G90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H86" s="10">
-        <f>SUM(G14:G83)</f>
-        <v>272.5</v>
-      </c>
-      <c r="J86" s="6" t="s">
+      <c r="H90" s="10">
+        <f>SUM(G14:G87)</f>
+        <v>327.5</v>
+      </c>
+      <c r="J90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K86" s="10">
-        <f>SUM(J14:J83)</f>
-        <v>-85</v>
-      </c>
-      <c r="M86" s="6" t="s">
+      <c r="K90" s="10">
+        <f>SUM(J14:J87)</f>
+        <v>-90</v>
+      </c>
+      <c r="M90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="N86" s="10">
-        <f>SUM(M14:M83)</f>
-        <v>-360</v>
-      </c>
-      <c r="P86" s="6" t="s">
+      <c r="N90" s="10">
+        <f>SUM(M14:M87)</f>
+        <v>-340</v>
+      </c>
+      <c r="P90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="Q86" s="10">
-        <f>SUM(P14:P83)</f>
-        <v>197.5</v>
-      </c>
-      <c r="S86" s="6" t="s">
+      <c r="Q90" s="10">
+        <f>SUM(P14:P87)</f>
+        <v>157.5</v>
+      </c>
+      <c r="S90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="T86" s="10">
-        <f>SUM(S14:S83)</f>
-        <v>145</v>
-      </c>
-      <c r="V86" s="6" t="s">
+      <c r="T90" s="10">
+        <f>SUM(S14:S87)</f>
+        <v>130</v>
+      </c>
+      <c r="V90" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="W86" s="10">
-        <f>SUM(V14:V83)</f>
-        <v>42.5</v>
-      </c>
-      <c r="Y86" s="17" t="s">
+      <c r="W90" s="10">
+        <f>SUM(V14:V87)</f>
+        <v>37.5</v>
+      </c>
+      <c r="Y90" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Z86" s="10">
-        <f>SUM(Y14:Y83)</f>
-        <v>-162.5</v>
-      </c>
-      <c r="AB86" s="17" t="s">
+      <c r="Z90" s="10">
+        <f>SUM(Y14:Y87)</f>
+        <v>-122.5</v>
+      </c>
+      <c r="AB90" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="AC86" s="10">
-        <f>SUM(AB14:AB83)</f>
-        <v>160</v>
-      </c>
-      <c r="AD86" s="1">
-        <f>SUM(E86,H86,K86,N86,Q86,T86,W86,Z86,AC86)</f>
+      <c r="AC90" s="10">
+        <f>SUM(AB14:AB87)</f>
+        <v>135</v>
+      </c>
+      <c r="AD90" s="1">
+        <f>SUM(E90,H90,K90,N90,Q90,T90,W90,Z90,AC90)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:30" ht="19" x14ac:dyDescent="0.25">
+      <c r="C96" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="D96" s="24"/>
+      <c r="E96" s="24"/>
+      <c r="F96" s="24"/>
+      <c r="G96" s="24"/>
+      <c r="H96" s="24"/>
+      <c r="I96" s="24"/>
+      <c r="J96" s="24"/>
+      <c r="O96" s="25"/>
+      <c r="P96" s="25"/>
+      <c r="R96" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="S96" s="26"/>
+      <c r="T96" s="26"/>
+      <c r="U96" s="26"/>
+      <c r="V96" s="26"/>
+      <c r="W96" s="25"/>
+    </row>
+    <row r="97" spans="2:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="C97" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="D97" s="24"/>
+      <c r="E97" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="F97" s="24"/>
+      <c r="G97" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="H97" s="24"/>
+      <c r="I97" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="J97" s="24"/>
+      <c r="O97" s="25"/>
+      <c r="P97" s="25"/>
+      <c r="R97" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="S97" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="T97" s="26"/>
+      <c r="U97" s="26"/>
+      <c r="V97" s="26"/>
+      <c r="W97" s="25"/>
+    </row>
+    <row r="98" spans="2:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="C98" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="D98" s="36"/>
+      <c r="E98" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="F98" s="36"/>
+      <c r="G98" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="H98" s="36"/>
+      <c r="I98" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="J98" s="36"/>
+      <c r="K98" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="R98" s="28"/>
+      <c r="S98" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="T98" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="U98" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="V98" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="W98" s="25"/>
+    </row>
+    <row r="99" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B99" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C99" s="37">
+        <v>0</v>
+      </c>
+      <c r="D99" s="38"/>
+      <c r="E99" s="37"/>
+      <c r="F99" s="38"/>
+      <c r="G99" s="37"/>
+      <c r="H99" s="38"/>
+      <c r="I99" s="37"/>
+      <c r="J99" s="38"/>
+      <c r="K99" s="14">
+        <f>SUM(C99:J99)</f>
+        <v>0</v>
+      </c>
+      <c r="Q99" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="R99" s="10">
+        <f>E90</f>
+        <v>-235</v>
+      </c>
+      <c r="S99" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T99" s="10">
+        <f>K99</f>
+        <v>0</v>
+      </c>
+      <c r="U99" s="10">
+        <f>IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T99, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V99" s="32">
+        <f>SUM(R99,S99,U99)</f>
+        <v>-635</v>
+      </c>
+      <c r="W99" s="14" t="str">
+        <f>Q99</f>
+        <v>Jaya</v>
+      </c>
+    </row>
+    <row r="100" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B100" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C100" s="37">
+        <v>5</v>
+      </c>
+      <c r="D100" s="38"/>
+      <c r="E100" s="37"/>
+      <c r="F100" s="38"/>
+      <c r="G100" s="37"/>
+      <c r="H100" s="38"/>
+      <c r="I100" s="37"/>
+      <c r="J100" s="38"/>
+      <c r="K100" s="14">
+        <f>SUM(C100:J100)</f>
+        <v>5</v>
+      </c>
+      <c r="Q100" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="R100" s="10">
+        <f>H90</f>
+        <v>327.5</v>
+      </c>
+      <c r="S100" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T100" s="10">
+        <f t="shared" ref="T100:T107" si="0">K100</f>
+        <v>5</v>
+      </c>
+      <c r="U100" s="10">
+        <f t="shared" ref="U100:U107" si="1">IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T100, 0)</f>
+        <v>1800</v>
+      </c>
+      <c r="V100" s="32">
+        <f t="shared" ref="V100:V106" si="2">SUM(R100,S100,U100)</f>
+        <v>1727.5</v>
+      </c>
+      <c r="W100" s="14" t="str">
+        <f t="shared" ref="W100:W106" si="3">Q100</f>
+        <v>Justin</v>
+      </c>
+    </row>
+    <row r="101" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B101" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C101" s="37">
+        <v>0</v>
+      </c>
+      <c r="D101" s="38"/>
+      <c r="E101" s="37"/>
+      <c r="F101" s="38"/>
+      <c r="G101" s="37"/>
+      <c r="H101" s="38"/>
+      <c r="I101" s="37"/>
+      <c r="J101" s="38"/>
+      <c r="K101" s="14">
+        <f>SUM(C101:J101)</f>
+        <v>0</v>
+      </c>
+      <c r="Q101" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="R101" s="10">
+        <f>K90</f>
+        <v>-90</v>
+      </c>
+      <c r="S101" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T101" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U101" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V101" s="32">
+        <f t="shared" si="2"/>
+        <v>-490</v>
+      </c>
+      <c r="W101" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Ram</v>
+      </c>
+    </row>
+    <row r="102" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B102" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C102" s="37">
+        <v>5</v>
+      </c>
+      <c r="D102" s="38"/>
+      <c r="E102" s="37"/>
+      <c r="F102" s="38"/>
+      <c r="G102" s="37"/>
+      <c r="H102" s="38"/>
+      <c r="I102" s="37"/>
+      <c r="J102" s="38"/>
+      <c r="K102" s="14">
+        <f>SUM(C102:J102)</f>
+        <v>5</v>
+      </c>
+      <c r="Q102" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="R102" s="10">
+        <f>N90</f>
+        <v>-340</v>
+      </c>
+      <c r="S102" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T102" s="10">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="U102" s="10">
+        <f t="shared" si="1"/>
+        <v>1800</v>
+      </c>
+      <c r="V102" s="32">
+        <f t="shared" si="2"/>
+        <v>1060</v>
+      </c>
+      <c r="W102" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Sibi</v>
+      </c>
+    </row>
+    <row r="103" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B103" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C103" s="37">
+        <v>0</v>
+      </c>
+      <c r="D103" s="38"/>
+      <c r="E103" s="37"/>
+      <c r="F103" s="38"/>
+      <c r="G103" s="37"/>
+      <c r="H103" s="38"/>
+      <c r="I103" s="37"/>
+      <c r="J103" s="38"/>
+      <c r="K103" s="14">
+        <f>SUM(C103:J103)</f>
+        <v>0</v>
+      </c>
+      <c r="Q103" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="R103" s="10">
+        <f>Q90</f>
+        <v>157.5</v>
+      </c>
+      <c r="S103" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T103" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U103" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V103" s="32">
+        <f t="shared" si="2"/>
+        <v>-242.5</v>
+      </c>
+      <c r="W103" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Sundar</v>
+      </c>
+    </row>
+    <row r="104" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B104" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C104" s="37">
+        <v>0</v>
+      </c>
+      <c r="D104" s="38"/>
+      <c r="E104" s="37"/>
+      <c r="F104" s="38"/>
+      <c r="G104" s="37"/>
+      <c r="H104" s="38"/>
+      <c r="I104" s="37"/>
+      <c r="J104" s="38"/>
+      <c r="K104" s="14">
+        <f>SUM(C104:J104)</f>
+        <v>0</v>
+      </c>
+      <c r="Q104" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="R104" s="10">
+        <f>T90</f>
+        <v>130</v>
+      </c>
+      <c r="S104" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T104" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U104" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V104" s="32">
+        <f t="shared" si="2"/>
+        <v>-270</v>
+      </c>
+      <c r="W104" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Rapaka</v>
+      </c>
+    </row>
+    <row r="105" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B105" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C105" s="37">
+        <v>0</v>
+      </c>
+      <c r="D105" s="38"/>
+      <c r="E105" s="37"/>
+      <c r="F105" s="38"/>
+      <c r="G105" s="37"/>
+      <c r="H105" s="38"/>
+      <c r="I105" s="37"/>
+      <c r="J105" s="38"/>
+      <c r="K105" s="14">
+        <f>SUM(C105:J105)</f>
+        <v>0</v>
+      </c>
+      <c r="Q105" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="R105" s="10">
+        <f>W90</f>
+        <v>37.5</v>
+      </c>
+      <c r="S105" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T105" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U105" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V105" s="32">
+        <f t="shared" si="2"/>
+        <v>-362.5</v>
+      </c>
+      <c r="W105" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Jayanth</v>
+      </c>
+    </row>
+    <row r="106" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B106" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C106" s="37">
+        <v>0</v>
+      </c>
+      <c r="D106" s="38"/>
+      <c r="E106" s="37"/>
+      <c r="F106" s="38"/>
+      <c r="G106" s="37"/>
+      <c r="H106" s="38"/>
+      <c r="I106" s="37"/>
+      <c r="J106" s="38"/>
+      <c r="K106" s="14">
+        <f>SUM(C106:J106)</f>
+        <v>0</v>
+      </c>
+      <c r="Q106" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="R106" s="10">
+        <f>Z90</f>
+        <v>-122.5</v>
+      </c>
+      <c r="S106" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T106" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U106" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V106" s="32">
+        <f t="shared" si="2"/>
+        <v>-522.5</v>
+      </c>
+      <c r="W106" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>Vicky</v>
+      </c>
+    </row>
+    <row r="107" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B107" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C107" s="37">
+        <v>0</v>
+      </c>
+      <c r="D107" s="38"/>
+      <c r="E107" s="37"/>
+      <c r="F107" s="38"/>
+      <c r="G107" s="37"/>
+      <c r="H107" s="38"/>
+      <c r="I107" s="37"/>
+      <c r="J107" s="38"/>
+      <c r="K107" s="14">
+        <f>SUM(C107:J107)</f>
+        <v>0</v>
+      </c>
+      <c r="Q107" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="R107" s="10">
+        <f>AC90</f>
+        <v>135</v>
+      </c>
+      <c r="S107" s="31">
+        <v>-400</v>
+      </c>
+      <c r="T107" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U107" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V107" s="32">
+        <f t="shared" ref="V107" si="4">SUM(R107,S107,U107)</f>
+        <v>-265</v>
+      </c>
+      <c r="W107" s="14" t="str">
+        <f t="shared" ref="W107" si="5">Q107</f>
+        <v>Anantha</v>
+      </c>
+    </row>
+    <row r="108" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="R108" s="33">
+        <f>SUM(R99:R107)</f>
+        <v>0</v>
+      </c>
+      <c r="V108" s="34">
+        <f>SUM(V99:V107)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
-  <mergeCells count="10">
+  <mergeCells count="58">
+    <mergeCell ref="I104:J104"/>
+    <mergeCell ref="I105:J105"/>
+    <mergeCell ref="I106:J106"/>
+    <mergeCell ref="I107:J107"/>
+    <mergeCell ref="E98:F98"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="I98:J98"/>
+    <mergeCell ref="I99:J99"/>
+    <mergeCell ref="I100:J100"/>
+    <mergeCell ref="I101:J101"/>
+    <mergeCell ref="I102:J102"/>
+    <mergeCell ref="I103:J103"/>
+    <mergeCell ref="E104:F104"/>
+    <mergeCell ref="E105:F105"/>
+    <mergeCell ref="E106:F106"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="G100:H100"/>
+    <mergeCell ref="G101:H101"/>
+    <mergeCell ref="G102:H102"/>
+    <mergeCell ref="G103:H103"/>
+    <mergeCell ref="G104:H104"/>
+    <mergeCell ref="G105:H105"/>
+    <mergeCell ref="G106:H106"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="E99:F99"/>
+    <mergeCell ref="E100:F100"/>
+    <mergeCell ref="E101:F101"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="E103:F103"/>
+    <mergeCell ref="C99:D99"/>
+    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="C101:D101"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C103:D103"/>
+    <mergeCell ref="C104:D104"/>
+    <mergeCell ref="C106:D106"/>
+    <mergeCell ref="C105:D105"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="C96:J96"/>
+    <mergeCell ref="R96:V96"/>
+    <mergeCell ref="C97:D97"/>
+    <mergeCell ref="E97:F97"/>
+    <mergeCell ref="G97:H97"/>
+    <mergeCell ref="I97:J97"/>
+    <mergeCell ref="R97:R98"/>
+    <mergeCell ref="S97:V97"/>
+    <mergeCell ref="C98:D98"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="I2:X9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="V12:W12"/>
     <mergeCell ref="Y12:Z12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="AB12:AC12"/>
   </mergeCells>
-  <conditionalFormatting sqref="E86">
-    <cfRule type="cellIs" dxfId="26" priority="246" operator="greaterThan">
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="E90">
+    <cfRule type="cellIs" dxfId="32" priority="274" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="245" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="275" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="244" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="276" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
+  <conditionalFormatting sqref="H90">
+    <cfRule type="cellIs" dxfId="29" priority="28" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="29" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="30" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K90">
+    <cfRule type="cellIs" dxfId="26" priority="25" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="26" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="27" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N90">
+    <cfRule type="cellIs" dxfId="23" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K86">
-    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
+  <conditionalFormatting sqref="Q90">
+    <cfRule type="cellIs" dxfId="20" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N86">
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="greaterThan">
+  <conditionalFormatting sqref="T90">
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q86">
-    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+  <conditionalFormatting sqref="W90">
+    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T86">
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
+  <conditionalFormatting sqref="Z90">
+    <cfRule type="cellIs" dxfId="11" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W86">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
+  <conditionalFormatting sqref="AC90">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z86">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+  <conditionalFormatting sqref="R99:R107">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC86">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+  <conditionalFormatting sqref="V99:V107">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Eliminator GT vs MI
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBDB813-A83D-1946-8501-AF3C5F6CC1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E982DE0-7B9B-FA44-A90A-C7B4D70D6A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="124">
   <si>
     <t>Points</t>
   </si>
@@ -6864,52 +6864,72 @@
       <c r="B85" s="4">
         <v>1</v>
       </c>
-      <c r="C85" s="18"/>
-      <c r="D85" s="3" t="str">
+      <c r="C85" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E85" s="4"/>
-      <c r="G85" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E85" s="4">
+        <v>100</v>
+      </c>
+      <c r="G85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H85" s="4"/>
-      <c r="J85" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="H85" s="4">
+        <v>70</v>
+      </c>
+      <c r="J85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K85" s="4"/>
-      <c r="M85" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K85" s="4">
+        <v>50</v>
+      </c>
+      <c r="M85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N85" s="4"/>
-      <c r="P85" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N85" s="4">
+        <v>0</v>
+      </c>
+      <c r="P85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q85" s="4"/>
-      <c r="S85" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q85" s="4">
+        <v>60</v>
+      </c>
+      <c r="S85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T85" s="4"/>
-      <c r="V85" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T85" s="4">
+        <v>30</v>
+      </c>
+      <c r="V85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W85" s="4"/>
-      <c r="Y85" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W85" s="4">
+        <v>90</v>
+      </c>
+      <c r="Y85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z85" s="4"/>
-      <c r="AB85" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z85" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85,$AC85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC85" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="AC85" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="86" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
@@ -6918,7 +6938,9 @@
       <c r="B86" s="4">
         <v>1</v>
       </c>
-      <c r="C86" s="18"/>
+      <c r="C86" s="18" t="s">
+        <v>106</v>
+      </c>
       <c r="D86" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -7115,7 +7137,7 @@
       </c>
       <c r="E90" s="10">
         <f>SUM(D14:D87)</f>
-        <v>-235</v>
+        <v>-185</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>7</v>
@@ -7129,49 +7151,49 @@
       </c>
       <c r="K90" s="10">
         <f>SUM(J14:J87)</f>
-        <v>-90</v>
+        <v>-100</v>
       </c>
       <c r="M90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N90" s="10">
         <f>SUM(M14:M87)</f>
-        <v>-340</v>
+        <v>-365</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q90" s="10">
         <f>SUM(P14:P87)</f>
-        <v>157.5</v>
+        <v>152.5</v>
       </c>
       <c r="S90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T90" s="10">
         <f>SUM(S14:S87)</f>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="V90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W90" s="10">
         <f>SUM(V14:V87)</f>
-        <v>37.5</v>
+        <v>57.5</v>
       </c>
       <c r="Y90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z90" s="10">
         <f>SUM(Y14:Y87)</f>
-        <v>-122.5</v>
+        <v>-117.5</v>
       </c>
       <c r="AB90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC90" s="10">
         <f>SUM(AB14:AB87)</f>
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="AD90" s="1">
         <f>SUM(E90,H90,K90,N90,Q90,T90,W90,Z90,AC90)</f>
@@ -7273,7 +7295,9 @@
         <v>0</v>
       </c>
       <c r="D99" s="38"/>
-      <c r="E99" s="37"/>
+      <c r="E99" s="37">
+        <v>3</v>
+      </c>
       <c r="F99" s="38"/>
       <c r="G99" s="37"/>
       <c r="H99" s="38"/>
@@ -7281,29 +7305,29 @@
       <c r="J99" s="38"/>
       <c r="K99" s="14">
         <f>SUM(C99:J99)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q99" s="14" t="s">
         <v>8</v>
       </c>
       <c r="R99" s="10">
         <f>E90</f>
-        <v>-235</v>
+        <v>-185</v>
       </c>
       <c r="S99" s="31">
         <v>-400</v>
       </c>
       <c r="T99" s="10">
         <f>K99</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U99" s="10">
         <f>IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T99, 0)</f>
-        <v>0</v>
+        <v>514.28571428571422</v>
       </c>
       <c r="V99" s="32">
         <f>SUM(R99,S99,U99)</f>
-        <v>-635</v>
+        <v>-70.714285714285779</v>
       </c>
       <c r="W99" s="14" t="str">
         <f>Q99</f>
@@ -7318,7 +7342,9 @@
         <v>5</v>
       </c>
       <c r="D100" s="38"/>
-      <c r="E100" s="37"/>
+      <c r="E100" s="37">
+        <v>0</v>
+      </c>
       <c r="F100" s="38"/>
       <c r="G100" s="37"/>
       <c r="H100" s="38"/>
@@ -7344,11 +7370,11 @@
       </c>
       <c r="U100" s="10">
         <f t="shared" ref="U100:U107" si="1">IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T100, 0)</f>
-        <v>1800</v>
+        <v>857.14285714285711</v>
       </c>
       <c r="V100" s="32">
         <f t="shared" ref="V100:V106" si="2">SUM(R100,S100,U100)</f>
-        <v>1727.5</v>
+        <v>784.64285714285711</v>
       </c>
       <c r="W100" s="14" t="str">
         <f t="shared" ref="W100:W106" si="3">Q100</f>
@@ -7363,7 +7389,9 @@
         <v>0</v>
       </c>
       <c r="D101" s="38"/>
-      <c r="E101" s="37"/>
+      <c r="E101" s="37">
+        <v>0</v>
+      </c>
       <c r="F101" s="38"/>
       <c r="G101" s="37"/>
       <c r="H101" s="38"/>
@@ -7378,7 +7406,7 @@
       </c>
       <c r="R101" s="10">
         <f>K90</f>
-        <v>-90</v>
+        <v>-100</v>
       </c>
       <c r="S101" s="31">
         <v>-400</v>
@@ -7393,7 +7421,7 @@
       </c>
       <c r="V101" s="32">
         <f t="shared" si="2"/>
-        <v>-490</v>
+        <v>-500</v>
       </c>
       <c r="W101" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7408,7 +7436,9 @@
         <v>5</v>
       </c>
       <c r="D102" s="38"/>
-      <c r="E102" s="37"/>
+      <c r="E102" s="37">
+        <v>0</v>
+      </c>
       <c r="F102" s="38"/>
       <c r="G102" s="37"/>
       <c r="H102" s="38"/>
@@ -7423,7 +7453,7 @@
       </c>
       <c r="R102" s="10">
         <f>N90</f>
-        <v>-340</v>
+        <v>-365</v>
       </c>
       <c r="S102" s="31">
         <v>-400</v>
@@ -7434,11 +7464,11 @@
       </c>
       <c r="U102" s="10">
         <f t="shared" si="1"/>
-        <v>1800</v>
+        <v>857.14285714285711</v>
       </c>
       <c r="V102" s="32">
         <f t="shared" si="2"/>
-        <v>1060</v>
+        <v>92.14285714285711</v>
       </c>
       <c r="W102" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7453,7 +7483,9 @@
         <v>0</v>
       </c>
       <c r="D103" s="38"/>
-      <c r="E103" s="37"/>
+      <c r="E103" s="37">
+        <v>0</v>
+      </c>
       <c r="F103" s="38"/>
       <c r="G103" s="37"/>
       <c r="H103" s="38"/>
@@ -7468,7 +7500,7 @@
       </c>
       <c r="R103" s="10">
         <f>Q90</f>
-        <v>157.5</v>
+        <v>152.5</v>
       </c>
       <c r="S103" s="31">
         <v>-400</v>
@@ -7483,7 +7515,7 @@
       </c>
       <c r="V103" s="32">
         <f t="shared" si="2"/>
-        <v>-242.5</v>
+        <v>-247.5</v>
       </c>
       <c r="W103" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7498,7 +7530,9 @@
         <v>0</v>
       </c>
       <c r="D104" s="38"/>
-      <c r="E104" s="37"/>
+      <c r="E104" s="37">
+        <v>0</v>
+      </c>
       <c r="F104" s="38"/>
       <c r="G104" s="37"/>
       <c r="H104" s="38"/>
@@ -7513,7 +7547,7 @@
       </c>
       <c r="R104" s="10">
         <f>T90</f>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="S104" s="31">
         <v>-400</v>
@@ -7528,7 +7562,7 @@
       </c>
       <c r="V104" s="32">
         <f t="shared" si="2"/>
-        <v>-270</v>
+        <v>-290</v>
       </c>
       <c r="W104" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7543,7 +7577,9 @@
         <v>0</v>
       </c>
       <c r="D105" s="38"/>
-      <c r="E105" s="37"/>
+      <c r="E105" s="37">
+        <v>3</v>
+      </c>
       <c r="F105" s="38"/>
       <c r="G105" s="37"/>
       <c r="H105" s="38"/>
@@ -7551,29 +7587,29 @@
       <c r="J105" s="38"/>
       <c r="K105" s="14">
         <f>SUM(C105:J105)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q105" s="14" t="s">
         <v>29</v>
       </c>
       <c r="R105" s="10">
         <f>W90</f>
-        <v>37.5</v>
+        <v>57.5</v>
       </c>
       <c r="S105" s="31">
         <v>-400</v>
       </c>
       <c r="T105" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U105" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>514.28571428571422</v>
       </c>
       <c r="V105" s="32">
         <f t="shared" si="2"/>
-        <v>-362.5</v>
+        <v>171.78571428571422</v>
       </c>
       <c r="W105" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7588,7 +7624,9 @@
         <v>0</v>
       </c>
       <c r="D106" s="38"/>
-      <c r="E106" s="37"/>
+      <c r="E106" s="37">
+        <v>5</v>
+      </c>
       <c r="F106" s="38"/>
       <c r="G106" s="37"/>
       <c r="H106" s="38"/>
@@ -7596,29 +7634,29 @@
       <c r="J106" s="38"/>
       <c r="K106" s="14">
         <f>SUM(C106:J106)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q106" s="14" t="s">
         <v>18</v>
       </c>
       <c r="R106" s="10">
         <f>Z90</f>
-        <v>-122.5</v>
+        <v>-117.5</v>
       </c>
       <c r="S106" s="31">
         <v>-400</v>
       </c>
       <c r="T106" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U106" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>857.14285714285711</v>
       </c>
       <c r="V106" s="32">
         <f t="shared" si="2"/>
-        <v>-522.5</v>
+        <v>339.64285714285711</v>
       </c>
       <c r="W106" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7633,7 +7671,9 @@
         <v>0</v>
       </c>
       <c r="D107" s="38"/>
-      <c r="E107" s="37"/>
+      <c r="E107" s="37">
+        <v>0</v>
+      </c>
       <c r="F107" s="38"/>
       <c r="G107" s="37"/>
       <c r="H107" s="38"/>
@@ -7648,7 +7688,7 @@
       </c>
       <c r="R107" s="10">
         <f>AC90</f>
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="S107" s="31">
         <v>-400</v>
@@ -7663,7 +7703,7 @@
       </c>
       <c r="V107" s="32">
         <f t="shared" ref="V107" si="4">SUM(R107,S107,U107)</f>
-        <v>-265</v>
+        <v>-280</v>
       </c>
       <c r="W107" s="14" t="str">
         <f t="shared" ref="W107" si="5">Q107</f>

</xml_diff>

<commit_message>
qualifier 2 PBKS vs MI
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E982DE0-7B9B-FA44-A90A-C7B4D70D6A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641EE81A-6D86-954C-9941-FB303EA87531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="124">
   <si>
     <t>Points</t>
   </si>
@@ -6941,51 +6941,69 @@
       <c r="C86" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="D86" s="3" t="str">
+      <c r="D86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E86" s="4"/>
-      <c r="G86" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E86" s="4">
+        <v>100</v>
+      </c>
+      <c r="G86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H86" s="4"/>
-      <c r="J86" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H86" s="4">
+        <v>50</v>
+      </c>
+      <c r="J86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K86" s="4"/>
-      <c r="M86" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K86" s="4">
+        <v>30</v>
+      </c>
+      <c r="M86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N86" s="4"/>
-      <c r="P86" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N86" s="4">
+        <v>60</v>
+      </c>
+      <c r="P86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q86" s="4"/>
-      <c r="S86" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="4">
+        <v>70</v>
+      </c>
+      <c r="S86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T86" s="4"/>
-      <c r="V86" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T86" s="4">
+        <v>90</v>
+      </c>
+      <c r="V86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W86" s="4"/>
-      <c r="Y86" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W86" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z86" s="4"/>
-      <c r="AB86" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z86" s="4">
+        <v>80</v>
+      </c>
+      <c r="AB86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86,$AC86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC86" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="AC86" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="87" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
@@ -6994,7 +7012,9 @@
       <c r="B87" s="4">
         <v>1</v>
       </c>
-      <c r="C87" s="18"/>
+      <c r="C87" s="18" t="s">
+        <v>70</v>
+      </c>
       <c r="D87" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -7137,28 +7157,28 @@
       </c>
       <c r="E90" s="10">
         <f>SUM(D14:D87)</f>
-        <v>-185</v>
+        <v>-135</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H90" s="10">
         <f>SUM(G14:G87)</f>
-        <v>327.5</v>
+        <v>317.5</v>
       </c>
       <c r="J90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K90" s="10">
         <f>SUM(J14:J87)</f>
-        <v>-100</v>
+        <v>-120</v>
       </c>
       <c r="M90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N90" s="10">
         <f>SUM(M14:M87)</f>
-        <v>-365</v>
+        <v>-370</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>7</v>
@@ -7172,28 +7192,28 @@
       </c>
       <c r="T90" s="10">
         <f>SUM(S14:S87)</f>
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="V90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W90" s="10">
         <f>SUM(V14:V87)</f>
-        <v>57.5</v>
+        <v>32.5</v>
       </c>
       <c r="Y90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z90" s="10">
         <f>SUM(Y14:Y87)</f>
-        <v>-117.5</v>
+        <v>-112.5</v>
       </c>
       <c r="AB90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC90" s="10">
         <f>SUM(AB14:AB87)</f>
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="AD90" s="1">
         <f>SUM(E90,H90,K90,N90,Q90,T90,W90,Z90,AC90)</f>
@@ -7299,35 +7319,37 @@
         <v>3</v>
       </c>
       <c r="F99" s="38"/>
-      <c r="G99" s="37"/>
+      <c r="G99" s="37">
+        <v>3</v>
+      </c>
       <c r="H99" s="38"/>
       <c r="I99" s="37"/>
       <c r="J99" s="38"/>
       <c r="K99" s="14">
         <f>SUM(C99:J99)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q99" s="14" t="s">
         <v>8</v>
       </c>
       <c r="R99" s="10">
         <f>E90</f>
-        <v>-185</v>
+        <v>-135</v>
       </c>
       <c r="S99" s="31">
         <v>-400</v>
       </c>
       <c r="T99" s="10">
         <f>K99</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U99" s="10">
         <f>IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T99, 0)</f>
-        <v>514.28571428571422</v>
+        <v>553.84615384615381</v>
       </c>
       <c r="V99" s="32">
         <f>SUM(R99,S99,U99)</f>
-        <v>-70.714285714285779</v>
+        <v>18.846153846153811</v>
       </c>
       <c r="W99" s="14" t="str">
         <f>Q99</f>
@@ -7346,7 +7368,9 @@
         <v>0</v>
       </c>
       <c r="F100" s="38"/>
-      <c r="G100" s="37"/>
+      <c r="G100" s="37">
+        <v>0</v>
+      </c>
       <c r="H100" s="38"/>
       <c r="I100" s="37"/>
       <c r="J100" s="38"/>
@@ -7359,7 +7383,7 @@
       </c>
       <c r="R100" s="10">
         <f>H90</f>
-        <v>327.5</v>
+        <v>317.5</v>
       </c>
       <c r="S100" s="31">
         <v>-400</v>
@@ -7370,11 +7394,11 @@
       </c>
       <c r="U100" s="10">
         <f t="shared" ref="U100:U107" si="1">IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T100, 0)</f>
-        <v>857.14285714285711</v>
+        <v>461.53846153846155</v>
       </c>
       <c r="V100" s="32">
         <f t="shared" ref="V100:V106" si="2">SUM(R100,S100,U100)</f>
-        <v>784.64285714285711</v>
+        <v>379.03846153846155</v>
       </c>
       <c r="W100" s="14" t="str">
         <f t="shared" ref="W100:W106" si="3">Q100</f>
@@ -7393,35 +7417,37 @@
         <v>0</v>
       </c>
       <c r="F101" s="38"/>
-      <c r="G101" s="37"/>
+      <c r="G101" s="37">
+        <v>3</v>
+      </c>
       <c r="H101" s="38"/>
       <c r="I101" s="37"/>
       <c r="J101" s="38"/>
       <c r="K101" s="14">
         <f>SUM(C101:J101)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q101" s="14" t="s">
         <v>9</v>
       </c>
       <c r="R101" s="10">
         <f>K90</f>
-        <v>-100</v>
+        <v>-120</v>
       </c>
       <c r="S101" s="31">
         <v>-400</v>
       </c>
       <c r="T101" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U101" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>276.92307692307691</v>
       </c>
       <c r="V101" s="32">
         <f t="shared" si="2"/>
-        <v>-500</v>
+        <v>-243.07692307692309</v>
       </c>
       <c r="W101" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7440,35 +7466,37 @@
         <v>0</v>
       </c>
       <c r="F102" s="38"/>
-      <c r="G102" s="37"/>
+      <c r="G102" s="37">
+        <v>3</v>
+      </c>
       <c r="H102" s="38"/>
       <c r="I102" s="37"/>
       <c r="J102" s="38"/>
       <c r="K102" s="14">
         <f>SUM(C102:J102)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q102" s="14" t="s">
         <v>12</v>
       </c>
       <c r="R102" s="10">
         <f>N90</f>
-        <v>-365</v>
+        <v>-370</v>
       </c>
       <c r="S102" s="31">
         <v>-400</v>
       </c>
       <c r="T102" s="10">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U102" s="10">
         <f t="shared" si="1"/>
-        <v>857.14285714285711</v>
+        <v>738.46153846153845</v>
       </c>
       <c r="V102" s="32">
         <f t="shared" si="2"/>
-        <v>92.14285714285711</v>
+        <v>-31.538461538461547</v>
       </c>
       <c r="W102" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7487,13 +7515,15 @@
         <v>0</v>
       </c>
       <c r="F103" s="38"/>
-      <c r="G103" s="37"/>
+      <c r="G103" s="37">
+        <v>3</v>
+      </c>
       <c r="H103" s="38"/>
       <c r="I103" s="37"/>
       <c r="J103" s="38"/>
       <c r="K103" s="14">
         <f>SUM(C103:J103)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q103" s="14" t="s">
         <v>10</v>
@@ -7507,15 +7537,15 @@
       </c>
       <c r="T103" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U103" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>276.92307692307691</v>
       </c>
       <c r="V103" s="32">
         <f t="shared" si="2"/>
-        <v>-247.5</v>
+        <v>29.423076923076906</v>
       </c>
       <c r="W103" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7534,35 +7564,37 @@
         <v>0</v>
       </c>
       <c r="F104" s="38"/>
-      <c r="G104" s="37"/>
+      <c r="G104" s="37">
+        <v>3</v>
+      </c>
       <c r="H104" s="38"/>
       <c r="I104" s="37"/>
       <c r="J104" s="38"/>
       <c r="K104" s="14">
         <f>SUM(C104:J104)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q104" s="14" t="s">
         <v>41</v>
       </c>
       <c r="R104" s="10">
         <f>T90</f>
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="S104" s="31">
         <v>-400</v>
       </c>
       <c r="T104" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U104" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>276.92307692307691</v>
       </c>
       <c r="V104" s="32">
         <f t="shared" si="2"/>
-        <v>-290</v>
+        <v>6.9230769230769056</v>
       </c>
       <c r="W104" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7581,7 +7613,9 @@
         <v>3</v>
       </c>
       <c r="F105" s="38"/>
-      <c r="G105" s="37"/>
+      <c r="G105" s="37">
+        <v>0</v>
+      </c>
       <c r="H105" s="38"/>
       <c r="I105" s="37"/>
       <c r="J105" s="38"/>
@@ -7594,7 +7628,7 @@
       </c>
       <c r="R105" s="10">
         <f>W90</f>
-        <v>57.5</v>
+        <v>32.5</v>
       </c>
       <c r="S105" s="31">
         <v>-400</v>
@@ -7605,11 +7639,11 @@
       </c>
       <c r="U105" s="10">
         <f t="shared" si="1"/>
-        <v>514.28571428571422</v>
+        <v>276.92307692307691</v>
       </c>
       <c r="V105" s="32">
         <f t="shared" si="2"/>
-        <v>171.78571428571422</v>
+        <v>-90.576923076923094</v>
       </c>
       <c r="W105" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7628,35 +7662,37 @@
         <v>5</v>
       </c>
       <c r="F106" s="38"/>
-      <c r="G106" s="37"/>
+      <c r="G106" s="37">
+        <v>3</v>
+      </c>
       <c r="H106" s="38"/>
       <c r="I106" s="37"/>
       <c r="J106" s="38"/>
       <c r="K106" s="14">
         <f>SUM(C106:J106)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q106" s="14" t="s">
         <v>18</v>
       </c>
       <c r="R106" s="10">
         <f>Z90</f>
-        <v>-117.5</v>
+        <v>-112.5</v>
       </c>
       <c r="S106" s="31">
         <v>-400</v>
       </c>
       <c r="T106" s="10">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U106" s="10">
         <f t="shared" si="1"/>
-        <v>857.14285714285711</v>
+        <v>738.46153846153845</v>
       </c>
       <c r="V106" s="32">
         <f t="shared" si="2"/>
-        <v>339.64285714285711</v>
+        <v>225.96153846153845</v>
       </c>
       <c r="W106" s="14" t="str">
         <f t="shared" si="3"/>
@@ -7675,7 +7711,9 @@
         <v>0</v>
       </c>
       <c r="F107" s="38"/>
-      <c r="G107" s="37"/>
+      <c r="G107" s="37">
+        <v>0</v>
+      </c>
       <c r="H107" s="38"/>
       <c r="I107" s="37"/>
       <c r="J107" s="38"/>
@@ -7688,7 +7726,7 @@
       </c>
       <c r="R107" s="10">
         <f>AC90</f>
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="S107" s="31">
         <v>-400</v>
@@ -7703,7 +7741,7 @@
       </c>
       <c r="V107" s="32">
         <f t="shared" ref="V107" si="4">SUM(R107,S107,U107)</f>
-        <v>-280</v>
+        <v>-295</v>
       </c>
       <c r="W107" s="14" t="str">
         <f t="shared" ref="W107" si="5">Q107</f>

</xml_diff>

<commit_message>
Finals - RCB won
</commit_message>
<xml_diff>
--- a/2025/NextGenIPLStandings2025.xlsx
+++ b/2025/NextGenIPLStandings2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641EE81A-6D86-954C-9941-FB303EA87531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B39E7FB-028B-AD49-866E-8767DC449B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="121">
   <si>
     <t>Points</t>
   </si>
@@ -405,15 +405,6 @@
   </si>
   <si>
     <t>Incoming</t>
-  </si>
-  <si>
-    <t>Format 3</t>
-  </si>
-  <si>
-    <t>Format 4</t>
-  </si>
-  <si>
-    <t>Format 5</t>
   </si>
 </sst>
 </file>
@@ -659,6 +650,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -672,30 +679,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -715,26 +706,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="33">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -887,6 +858,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -912,6 +903,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1007,6 +1008,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1022,26 +1033,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1064,9 +1055,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1104,7 +1095,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1210,7 +1201,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1352,7 +1343,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1393,24 +1384,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
-      <c r="S2" s="20"/>
-      <c r="T2" s="20"/>
-      <c r="U2" s="20"/>
-      <c r="V2" s="20"/>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="28"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="28"/>
     </row>
     <row r="3" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1419,22 +1410,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="20"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20"/>
-      <c r="T3" s="20"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
     </row>
     <row r="4" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1443,22 +1434,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="28"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="28"/>
+      <c r="U4" s="28"/>
+      <c r="V4" s="28"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
     </row>
     <row r="5" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1467,22 +1458,22 @@
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20"/>
-      <c r="T5" s="20"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+      <c r="U5" s="28"/>
+      <c r="V5" s="28"/>
+      <c r="W5" s="28"/>
+      <c r="X5" s="28"/>
     </row>
     <row r="6" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1491,22 +1482,22 @@
       <c r="B6" s="1">
         <v>-5</v>
       </c>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
-      <c r="T6" s="20"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="28"/>
+      <c r="U6" s="28"/>
+      <c r="V6" s="28"/>
+      <c r="W6" s="28"/>
+      <c r="X6" s="28"/>
     </row>
     <row r="7" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1515,22 +1506,22 @@
       <c r="B7" s="1">
         <v>-10</v>
       </c>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="20"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="20"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="20"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
+      <c r="U7" s="28"/>
+      <c r="V7" s="28"/>
+      <c r="W7" s="28"/>
+      <c r="X7" s="28"/>
     </row>
     <row r="8" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1539,22 +1530,22 @@
       <c r="B8" s="1">
         <v>-15</v>
       </c>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-      <c r="T8" s="20"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
+      <c r="R8" s="28"/>
+      <c r="S8" s="28"/>
+      <c r="T8" s="28"/>
+      <c r="U8" s="28"/>
+      <c r="V8" s="28"/>
+      <c r="W8" s="28"/>
+      <c r="X8" s="28"/>
     </row>
     <row r="9" spans="1:29" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1563,22 +1554,22 @@
       <c r="B9" s="1">
         <v>-20</v>
       </c>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
-      <c r="T9" s="20"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28"/>
+      <c r="T9" s="28"/>
+      <c r="U9" s="28"/>
+      <c r="V9" s="28"/>
+      <c r="W9" s="28"/>
+      <c r="X9" s="28"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1593,42 +1584,42 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="23"/>
-      <c r="G12" s="21" t="s">
+      <c r="E12" s="31"/>
+      <c r="G12" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="22"/>
-      <c r="J12" s="21" t="s">
+      <c r="H12" s="30"/>
+      <c r="J12" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="K12" s="22"/>
-      <c r="M12" s="21" t="s">
+      <c r="K12" s="30"/>
+      <c r="M12" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="N12" s="22"/>
-      <c r="P12" s="21" t="s">
+      <c r="N12" s="30"/>
+      <c r="P12" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="Q12" s="22"/>
-      <c r="S12" s="21" t="s">
+      <c r="Q12" s="30"/>
+      <c r="S12" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="T12" s="22"/>
-      <c r="V12" s="21" t="s">
+      <c r="T12" s="30"/>
+      <c r="V12" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="W12" s="22"/>
-      <c r="Y12" s="21" t="s">
+      <c r="W12" s="30"/>
+      <c r="Y12" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="Z12" s="22"/>
-      <c r="AB12" s="21" t="s">
+      <c r="Z12" s="30"/>
+      <c r="AB12" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="AC12" s="22"/>
+      <c r="AC12" s="30"/>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
@@ -7015,51 +7006,69 @@
       <c r="C87" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D87" s="3" t="str">
+      <c r="D87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E87" s="4"/>
-      <c r="G87" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E87" s="4">
+        <v>80</v>
+      </c>
+      <c r="G87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H87" s="4"/>
-      <c r="J87" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H87" s="4">
+        <v>60</v>
+      </c>
+      <c r="J87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K87" s="4"/>
-      <c r="M87" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K87" s="4">
+        <v>50</v>
+      </c>
+      <c r="M87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N87" s="4"/>
-      <c r="P87" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="N87" s="4">
+        <v>70</v>
+      </c>
+      <c r="P87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q87" s="4"/>
-      <c r="S87" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q87" s="4">
+        <v>30</v>
+      </c>
+      <c r="S87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T87" s="4"/>
-      <c r="V87" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T87" s="4">
+        <v>90</v>
+      </c>
+      <c r="V87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W87" s="4"/>
-      <c r="Y87" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W87" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z87" s="4"/>
-      <c r="AB87" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Z87" s="4">
+        <v>100</v>
+      </c>
+      <c r="AB87" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(AC87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(AC87, ($Z87,$W87,$T87,$Q87,$N87,$K87,$H87,$E87,$AC87), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="AC87" s="4"/>
+        <v>-25</v>
+      </c>
+      <c r="AC87" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="88" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A88" s="5"/>
@@ -7157,21 +7166,21 @@
       </c>
       <c r="E90" s="10">
         <f>SUM(D14:D87)</f>
-        <v>-135</v>
+        <v>-130</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H90" s="10">
         <f>SUM(G14:G87)</f>
-        <v>317.5</v>
+        <v>312.5</v>
       </c>
       <c r="J90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K90" s="10">
         <f>SUM(J14:J87)</f>
-        <v>-120</v>
+        <v>-130</v>
       </c>
       <c r="M90" s="6" t="s">
         <v>7</v>
@@ -7185,35 +7194,35 @@
       </c>
       <c r="Q90" s="10">
         <f>SUM(P14:P87)</f>
-        <v>152.5</v>
+        <v>132.5</v>
       </c>
       <c r="S90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T90" s="10">
         <f>SUM(S14:S87)</f>
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="V90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W90" s="10">
         <f>SUM(V14:V87)</f>
-        <v>32.5</v>
+        <v>17.5</v>
       </c>
       <c r="Y90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="Z90" s="10">
         <f>SUM(Y14:Y87)</f>
-        <v>-112.5</v>
+        <v>-62.5</v>
       </c>
       <c r="AB90" s="17" t="s">
         <v>7</v>
       </c>
       <c r="AC90" s="10">
         <f>SUM(AB14:AB87)</f>
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="AD90" s="1">
         <f>SUM(E90,H90,K90,N90,Q90,T90,W90,Z90,AC90)</f>
@@ -7221,56 +7230,56 @@
       </c>
     </row>
     <row r="96" spans="1:30" ht="19" x14ac:dyDescent="0.25">
-      <c r="C96" s="24" t="s">
+      <c r="C96" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="D96" s="24"/>
-      <c r="E96" s="24"/>
-      <c r="F96" s="24"/>
-      <c r="G96" s="24"/>
-      <c r="H96" s="24"/>
-      <c r="I96" s="24"/>
-      <c r="J96" s="24"/>
-      <c r="O96" s="25"/>
-      <c r="P96" s="25"/>
-      <c r="R96" s="26" t="s">
+      <c r="D96" s="33"/>
+      <c r="E96" s="33"/>
+      <c r="F96" s="33"/>
+      <c r="G96" s="33"/>
+      <c r="H96" s="33"/>
+      <c r="I96" s="33"/>
+      <c r="J96" s="33"/>
+      <c r="O96" s="20"/>
+      <c r="P96" s="20"/>
+      <c r="R96" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="S96" s="26"/>
-      <c r="T96" s="26"/>
-      <c r="U96" s="26"/>
-      <c r="V96" s="26"/>
-      <c r="W96" s="25"/>
+      <c r="S96" s="32"/>
+      <c r="T96" s="32"/>
+      <c r="U96" s="32"/>
+      <c r="V96" s="32"/>
+      <c r="W96" s="20"/>
     </row>
     <row r="97" spans="2:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="C97" s="24" t="s">
+      <c r="C97" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="D97" s="24"/>
-      <c r="E97" s="24" t="s">
+      <c r="D97" s="33"/>
+      <c r="E97" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="F97" s="24"/>
-      <c r="G97" s="24" t="s">
+      <c r="F97" s="33"/>
+      <c r="G97" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="H97" s="24"/>
-      <c r="I97" s="24" t="s">
+      <c r="H97" s="33"/>
+      <c r="I97" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="J97" s="24"/>
-      <c r="O97" s="25"/>
-      <c r="P97" s="25"/>
-      <c r="R97" s="26" t="s">
+      <c r="J97" s="33"/>
+      <c r="O97" s="20"/>
+      <c r="P97" s="20"/>
+      <c r="R97" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="S97" s="26" t="s">
+      <c r="S97" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="T97" s="26"/>
-      <c r="U97" s="26"/>
-      <c r="V97" s="26"/>
-      <c r="W97" s="25"/>
+      <c r="T97" s="32"/>
+      <c r="U97" s="32"/>
+      <c r="V97" s="32"/>
+      <c r="W97" s="20"/>
     </row>
     <row r="98" spans="2:23" ht="19" x14ac:dyDescent="0.25">
       <c r="C98" s="35" t="s">
@@ -7278,37 +7287,37 @@
       </c>
       <c r="D98" s="36"/>
       <c r="E98" s="35" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F98" s="36"/>
       <c r="G98" s="35" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="H98" s="36"/>
       <c r="I98" s="35" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J98" s="36"/>
-      <c r="K98" s="27" t="s">
+      <c r="K98" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="R98" s="28"/>
-      <c r="S98" s="29" t="s">
+      <c r="R98" s="34"/>
+      <c r="S98" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="T98" s="29" t="s">
+      <c r="T98" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="U98" s="29" t="s">
+      <c r="U98" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="V98" s="29" t="s">
+      <c r="V98" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="W98" s="25"/>
+      <c r="W98" s="20"/>
     </row>
     <row r="99" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B99" s="30" t="s">
+      <c r="B99" s="23" t="s">
         <v>8</v>
       </c>
       <c r="C99" s="37">
@@ -7323,10 +7332,12 @@
         <v>3</v>
       </c>
       <c r="H99" s="38"/>
-      <c r="I99" s="37"/>
+      <c r="I99" s="37">
+        <v>0</v>
+      </c>
       <c r="J99" s="38"/>
       <c r="K99" s="14">
-        <f>SUM(C99:J99)</f>
+        <f t="shared" ref="K99:K107" si="0">SUM(C99:J99)</f>
         <v>6</v>
       </c>
       <c r="Q99" s="14" t="s">
@@ -7334,9 +7345,9 @@
       </c>
       <c r="R99" s="10">
         <f>E90</f>
-        <v>-135</v>
-      </c>
-      <c r="S99" s="31">
+        <v>-130</v>
+      </c>
+      <c r="S99" s="24">
         <v>-400</v>
       </c>
       <c r="T99" s="10">
@@ -7347,9 +7358,9 @@
         <f>IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T99, 0)</f>
         <v>553.84615384615381</v>
       </c>
-      <c r="V99" s="32">
+      <c r="V99" s="25">
         <f>SUM(R99,S99,U99)</f>
-        <v>18.846153846153811</v>
+        <v>23.846153846153811</v>
       </c>
       <c r="W99" s="14" t="str">
         <f>Q99</f>
@@ -7357,7 +7368,7 @@
       </c>
     </row>
     <row r="100" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B100" s="30" t="s">
+      <c r="B100" s="23" t="s">
         <v>5</v>
       </c>
       <c r="C100" s="37">
@@ -7372,10 +7383,12 @@
         <v>0</v>
       </c>
       <c r="H100" s="38"/>
-      <c r="I100" s="37"/>
+      <c r="I100" s="37">
+        <v>0</v>
+      </c>
       <c r="J100" s="38"/>
       <c r="K100" s="14">
-        <f>SUM(C100:J100)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="Q100" s="14" t="s">
@@ -7383,30 +7396,30 @@
       </c>
       <c r="R100" s="10">
         <f>H90</f>
-        <v>317.5</v>
-      </c>
-      <c r="S100" s="31">
+        <v>312.5</v>
+      </c>
+      <c r="S100" s="24">
         <v>-400</v>
       </c>
       <c r="T100" s="10">
-        <f t="shared" ref="T100:T107" si="0">K100</f>
+        <f t="shared" ref="T100:T107" si="1">K100</f>
         <v>5</v>
       </c>
       <c r="U100" s="10">
-        <f t="shared" ref="U100:U107" si="1">IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T100, 0)</f>
+        <f t="shared" ref="U100:U107" si="2">IFERROR((-SUM($S$99:$S$107)/SUM($T$99:$T$107))*$T100, 0)</f>
         <v>461.53846153846155</v>
       </c>
-      <c r="V100" s="32">
-        <f t="shared" ref="V100:V106" si="2">SUM(R100,S100,U100)</f>
-        <v>379.03846153846155</v>
+      <c r="V100" s="25">
+        <f t="shared" ref="V100:V106" si="3">SUM(R100,S100,U100)</f>
+        <v>374.03846153846155</v>
       </c>
       <c r="W100" s="14" t="str">
-        <f t="shared" ref="W100:W106" si="3">Q100</f>
+        <f t="shared" ref="W100:W106" si="4">Q100</f>
         <v>Justin</v>
       </c>
     </row>
     <row r="101" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B101" s="30" t="s">
+      <c r="B101" s="23" t="s">
         <v>9</v>
       </c>
       <c r="C101" s="37">
@@ -7421,10 +7434,12 @@
         <v>3</v>
       </c>
       <c r="H101" s="38"/>
-      <c r="I101" s="37"/>
+      <c r="I101" s="37">
+        <v>0</v>
+      </c>
       <c r="J101" s="38"/>
       <c r="K101" s="14">
-        <f>SUM(C101:J101)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="Q101" s="14" t="s">
@@ -7432,30 +7447,30 @@
       </c>
       <c r="R101" s="10">
         <f>K90</f>
-        <v>-120</v>
-      </c>
-      <c r="S101" s="31">
+        <v>-130</v>
+      </c>
+      <c r="S101" s="24">
         <v>-400</v>
       </c>
       <c r="T101" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="U101" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>276.92307692307691</v>
       </c>
-      <c r="V101" s="32">
-        <f t="shared" si="2"/>
-        <v>-243.07692307692309</v>
+      <c r="V101" s="25">
+        <f t="shared" si="3"/>
+        <v>-253.07692307692309</v>
       </c>
       <c r="W101" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Ram</v>
       </c>
     </row>
     <row r="102" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B102" s="30" t="s">
+      <c r="B102" s="23" t="s">
         <v>12</v>
       </c>
       <c r="C102" s="37">
@@ -7470,10 +7485,12 @@
         <v>3</v>
       </c>
       <c r="H102" s="38"/>
-      <c r="I102" s="37"/>
+      <c r="I102" s="37">
+        <v>0</v>
+      </c>
       <c r="J102" s="38"/>
       <c r="K102" s="14">
-        <f>SUM(C102:J102)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="Q102" s="14" t="s">
@@ -7483,28 +7500,28 @@
         <f>N90</f>
         <v>-370</v>
       </c>
-      <c r="S102" s="31">
+      <c r="S102" s="24">
         <v>-400</v>
       </c>
       <c r="T102" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="U102" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>738.46153846153845</v>
       </c>
-      <c r="V102" s="32">
-        <f t="shared" si="2"/>
+      <c r="V102" s="25">
+        <f t="shared" si="3"/>
         <v>-31.538461538461547</v>
       </c>
       <c r="W102" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Sibi</v>
       </c>
     </row>
     <row r="103" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B103" s="30" t="s">
+      <c r="B103" s="23" t="s">
         <v>10</v>
       </c>
       <c r="C103" s="37">
@@ -7519,10 +7536,12 @@
         <v>3</v>
       </c>
       <c r="H103" s="38"/>
-      <c r="I103" s="37"/>
+      <c r="I103" s="37">
+        <v>0</v>
+      </c>
       <c r="J103" s="38"/>
       <c r="K103" s="14">
-        <f>SUM(C103:J103)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="Q103" s="14" t="s">
@@ -7530,30 +7549,30 @@
       </c>
       <c r="R103" s="10">
         <f>Q90</f>
-        <v>152.5</v>
-      </c>
-      <c r="S103" s="31">
+        <v>132.5</v>
+      </c>
+      <c r="S103" s="24">
         <v>-400</v>
       </c>
       <c r="T103" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="U103" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>276.92307692307691</v>
       </c>
-      <c r="V103" s="32">
-        <f t="shared" si="2"/>
-        <v>29.423076923076906</v>
+      <c r="V103" s="25">
+        <f t="shared" si="3"/>
+        <v>9.4230769230769056</v>
       </c>
       <c r="W103" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Sundar</v>
       </c>
     </row>
     <row r="104" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B104" s="30" t="s">
+      <c r="B104" s="23" t="s">
         <v>41</v>
       </c>
       <c r="C104" s="37">
@@ -7568,10 +7587,12 @@
         <v>3</v>
       </c>
       <c r="H104" s="38"/>
-      <c r="I104" s="37"/>
+      <c r="I104" s="37">
+        <v>0</v>
+      </c>
       <c r="J104" s="38"/>
       <c r="K104" s="14">
-        <f>SUM(C104:J104)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="Q104" s="14" t="s">
@@ -7579,30 +7600,30 @@
       </c>
       <c r="R104" s="10">
         <f>T90</f>
-        <v>130</v>
-      </c>
-      <c r="S104" s="31">
+        <v>150</v>
+      </c>
+      <c r="S104" s="24">
         <v>-400</v>
       </c>
       <c r="T104" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="U104" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>276.92307692307691</v>
       </c>
-      <c r="V104" s="32">
-        <f t="shared" si="2"/>
-        <v>6.9230769230769056</v>
+      <c r="V104" s="25">
+        <f t="shared" si="3"/>
+        <v>26.923076923076906</v>
       </c>
       <c r="W104" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Rapaka</v>
       </c>
     </row>
     <row r="105" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B105" s="30" t="s">
+      <c r="B105" s="23" t="s">
         <v>29</v>
       </c>
       <c r="C105" s="37">
@@ -7617,10 +7638,12 @@
         <v>0</v>
       </c>
       <c r="H105" s="38"/>
-      <c r="I105" s="37"/>
+      <c r="I105" s="37">
+        <v>0</v>
+      </c>
       <c r="J105" s="38"/>
       <c r="K105" s="14">
-        <f>SUM(C105:J105)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="Q105" s="14" t="s">
@@ -7628,30 +7651,30 @@
       </c>
       <c r="R105" s="10">
         <f>W90</f>
-        <v>32.5</v>
-      </c>
-      <c r="S105" s="31">
+        <v>17.5</v>
+      </c>
+      <c r="S105" s="24">
         <v>-400</v>
       </c>
       <c r="T105" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="U105" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>276.92307692307691</v>
       </c>
-      <c r="V105" s="32">
-        <f t="shared" si="2"/>
-        <v>-90.576923076923094</v>
+      <c r="V105" s="25">
+        <f t="shared" si="3"/>
+        <v>-105.57692307692309</v>
       </c>
       <c r="W105" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Jayanth</v>
       </c>
     </row>
     <row r="106" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B106" s="30" t="s">
+      <c r="B106" s="23" t="s">
         <v>18</v>
       </c>
       <c r="C106" s="37">
@@ -7666,10 +7689,12 @@
         <v>3</v>
       </c>
       <c r="H106" s="38"/>
-      <c r="I106" s="37"/>
+      <c r="I106" s="37">
+        <v>0</v>
+      </c>
       <c r="J106" s="38"/>
       <c r="K106" s="14">
-        <f>SUM(C106:J106)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="Q106" s="14" t="s">
@@ -7677,30 +7702,30 @@
       </c>
       <c r="R106" s="10">
         <f>Z90</f>
-        <v>-112.5</v>
-      </c>
-      <c r="S106" s="31">
+        <v>-62.5</v>
+      </c>
+      <c r="S106" s="24">
         <v>-400</v>
       </c>
       <c r="T106" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="U106" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>738.46153846153845</v>
       </c>
-      <c r="V106" s="32">
-        <f t="shared" si="2"/>
-        <v>225.96153846153845</v>
+      <c r="V106" s="25">
+        <f t="shared" si="3"/>
+        <v>275.96153846153845</v>
       </c>
       <c r="W106" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Vicky</v>
       </c>
     </row>
     <row r="107" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="B107" s="30" t="s">
+      <c r="B107" s="23" t="s">
         <v>44</v>
       </c>
       <c r="C107" s="37">
@@ -7715,10 +7740,12 @@
         <v>0</v>
       </c>
       <c r="H107" s="38"/>
-      <c r="I107" s="37"/>
+      <c r="I107" s="37">
+        <v>0</v>
+      </c>
       <c r="J107" s="38"/>
       <c r="K107" s="14">
-        <f>SUM(C107:J107)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q107" s="14" t="s">
@@ -7726,34 +7753,34 @@
       </c>
       <c r="R107" s="10">
         <f>AC90</f>
-        <v>105</v>
-      </c>
-      <c r="S107" s="31">
+        <v>80</v>
+      </c>
+      <c r="S107" s="24">
         <v>-400</v>
       </c>
       <c r="T107" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U107" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="V107" s="32">
-        <f t="shared" ref="V107" si="4">SUM(R107,S107,U107)</f>
-        <v>-295</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V107" s="25">
+        <f t="shared" ref="V107" si="5">SUM(R107,S107,U107)</f>
+        <v>-320</v>
       </c>
       <c r="W107" s="14" t="str">
-        <f t="shared" ref="W107" si="5">Q107</f>
+        <f t="shared" ref="W107" si="6">Q107</f>
         <v>Anantha</v>
       </c>
     </row>
     <row r="108" spans="2:23" ht="21" x14ac:dyDescent="0.25">
-      <c r="R108" s="33">
+      <c r="R108" s="26">
         <f>SUM(R99:R107)</f>
         <v>0</v>
       </c>
-      <c r="V108" s="34">
+      <c r="V108" s="27">
         <f>SUM(V99:V107)</f>
         <v>0</v>
       </c>
@@ -7777,30 +7804,30 @@
     <mergeCell ref="E105:F105"/>
     <mergeCell ref="E106:F106"/>
     <mergeCell ref="E107:F107"/>
+    <mergeCell ref="E101:F101"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="E103:F103"/>
     <mergeCell ref="G99:H99"/>
     <mergeCell ref="G100:H100"/>
     <mergeCell ref="G101:H101"/>
     <mergeCell ref="G102:H102"/>
     <mergeCell ref="G103:H103"/>
+    <mergeCell ref="C104:D104"/>
+    <mergeCell ref="C106:D106"/>
+    <mergeCell ref="C105:D105"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="C96:J96"/>
+    <mergeCell ref="C99:D99"/>
+    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="C101:D101"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C103:D103"/>
     <mergeCell ref="G104:H104"/>
     <mergeCell ref="G105:H105"/>
     <mergeCell ref="G106:H106"/>
     <mergeCell ref="G107:H107"/>
     <mergeCell ref="E99:F99"/>
     <mergeCell ref="E100:F100"/>
-    <mergeCell ref="E101:F101"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="C99:D99"/>
-    <mergeCell ref="C100:D100"/>
-    <mergeCell ref="C101:D101"/>
-    <mergeCell ref="C102:D102"/>
-    <mergeCell ref="C103:D103"/>
-    <mergeCell ref="C104:D104"/>
-    <mergeCell ref="C106:D106"/>
-    <mergeCell ref="C105:D105"/>
-    <mergeCell ref="C107:D107"/>
-    <mergeCell ref="C96:J96"/>
     <mergeCell ref="R96:V96"/>
     <mergeCell ref="C97:D97"/>
     <mergeCell ref="E97:F97"/>
@@ -7822,10 +7849,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E90">
-    <cfRule type="cellIs" dxfId="32" priority="274" operator="lessThan">
+    <cfRule type="cellIs" dxfId="32" priority="275" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="275" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="274" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="30" priority="276" operator="greaterThan">
@@ -7833,35 +7860,35 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H90">
-    <cfRule type="cellIs" dxfId="29" priority="28" operator="lessThan">
+    <cfRule type="cellIs" dxfId="29" priority="30" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="28" priority="29" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="30" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="28" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K90">
-    <cfRule type="cellIs" dxfId="26" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N90">
-    <cfRule type="cellIs" dxfId="23" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7869,76 +7896,76 @@
     <cfRule type="cellIs" dxfId="20" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R99:R107">
+    <cfRule type="cellIs" dxfId="17" priority="4" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="5" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T90">
-    <cfRule type="cellIs" dxfId="17" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="16" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V99:V107">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W90">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="14" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="13" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z90">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="10" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC90">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R99:R107">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V99:V107">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>